<commit_message>
update penyaluran dan perubahan format excel
</commit_message>
<xml_diff>
--- a/laporan_maal.xlsx
+++ b/laporan_maal.xlsx
@@ -1129,27 +1129,27 @@
       </c>
       <c r="B6" s="40" t="inlineStr">
         <is>
-          <t>2026-03-10</t>
+          <t>2026-03-20</t>
         </is>
       </c>
       <c r="C6" s="40" t="inlineStr">
         <is>
-          <t>21:13</t>
+          <t>15:37</t>
         </is>
       </c>
       <c r="D6" s="40" t="inlineStr">
         <is>
-          <t>Budi Rizki</t>
+          <t>INDRA ZAKI RAMADANI</t>
         </is>
       </c>
       <c r="E6" s="40" t="inlineStr">
         <is>
-          <t>Tipar Kidul</t>
+          <t>Ajibarang Wetan</t>
         </is>
       </c>
       <c r="F6" s="41" t="inlineStr">
         <is>
-          <t>01</t>
+          <t>02</t>
         </is>
       </c>
       <c r="G6" s="41" t="inlineStr">
@@ -1159,16 +1159,16 @@
       </c>
       <c r="H6" s="41" t="inlineStr">
         <is>
-          <t>instansi</t>
+          <t>perorangan</t>
         </is>
       </c>
       <c r="I6" s="40" t="inlineStr">
         <is>
-          <t>Shodaqoh</t>
+          <t>Zakat Maal</t>
         </is>
       </c>
       <c r="J6" s="41" t="n">
-        <v>50000</v>
+        <v>100000</v>
       </c>
       <c r="K6" s="8" t="n"/>
       <c r="L6" s="9" t="n"/>
@@ -1181,27 +1181,27 @@
       </c>
       <c r="B7" s="42" t="inlineStr">
         <is>
-          <t>2026-03-10</t>
+          <t>2026-03-20</t>
         </is>
       </c>
       <c r="C7" s="42" t="inlineStr">
         <is>
-          <t>20:37</t>
+          <t>16:05</t>
         </is>
       </c>
       <c r="D7" s="42" t="inlineStr">
         <is>
-          <t>Dedi Umar</t>
+          <t>INDRA ZAKI RAMADANI</t>
         </is>
       </c>
       <c r="E7" s="42" t="inlineStr">
         <is>
-          <t>Tipar Lor</t>
+          <t>Ajibarang Wetan</t>
         </is>
       </c>
       <c r="F7" s="42" t="inlineStr">
         <is>
-          <t>01</t>
+          <t>02</t>
         </is>
       </c>
       <c r="G7" s="42" t="inlineStr">
@@ -1211,7 +1211,7 @@
       </c>
       <c r="H7" s="42" t="inlineStr">
         <is>
-          <t>instansi</t>
+          <t>perorangan</t>
         </is>
       </c>
       <c r="I7" s="43" t="inlineStr">
@@ -1226,102 +1226,30 @@
       <c r="L7" s="45" t="n"/>
     </row>
     <row r="8" ht="15" customHeight="1" s="16">
-      <c r="A8" s="42" t="n">
-        <v>3</v>
-      </c>
-      <c r="B8" s="42" t="inlineStr">
-        <is>
-          <t>2026-03-03</t>
-        </is>
-      </c>
-      <c r="C8" s="42" t="inlineStr">
-        <is>
-          <t>17:40</t>
-        </is>
-      </c>
-      <c r="D8" s="42" t="inlineStr">
-        <is>
-          <t>Eko Fajar</t>
-        </is>
-      </c>
-      <c r="E8" s="42" t="inlineStr">
-        <is>
-          <t>Tipar Lor</t>
-        </is>
-      </c>
-      <c r="F8" s="42" t="inlineStr">
-        <is>
-          <t>01</t>
-        </is>
-      </c>
-      <c r="G8" s="42" t="inlineStr">
-        <is>
-          <t>01</t>
-        </is>
-      </c>
-      <c r="H8" s="42" t="inlineStr">
-        <is>
-          <t>perorangan</t>
-        </is>
-      </c>
-      <c r="I8" s="43" t="inlineStr">
-        <is>
-          <t>Shodaqoh</t>
-        </is>
-      </c>
-      <c r="J8" s="44" t="n">
-        <v>100000</v>
-      </c>
+      <c r="A8" s="42" t="n"/>
+      <c r="B8" s="42" t="n"/>
+      <c r="C8" s="42" t="n"/>
+      <c r="D8" s="42" t="n"/>
+      <c r="E8" s="42" t="n"/>
+      <c r="F8" s="42" t="n"/>
+      <c r="G8" s="42" t="n"/>
+      <c r="H8" s="42" t="n"/>
+      <c r="I8" s="43" t="n"/>
+      <c r="J8" s="44" t="n"/>
       <c r="K8" s="10" t="n"/>
       <c r="L8" s="45" t="n"/>
     </row>
     <row r="9" ht="15" customHeight="1" s="16">
-      <c r="A9" s="42" t="n">
-        <v>4</v>
-      </c>
-      <c r="B9" s="42" t="inlineStr">
-        <is>
-          <t>2026-03-11</t>
-        </is>
-      </c>
-      <c r="C9" s="42" t="inlineStr">
-        <is>
-          <t>17:40</t>
-        </is>
-      </c>
-      <c r="D9" s="42" t="inlineStr">
-        <is>
-          <t>Naufal Budi</t>
-        </is>
-      </c>
-      <c r="E9" s="42" t="inlineStr">
-        <is>
-          <t>Ajibarang Kulon</t>
-        </is>
-      </c>
-      <c r="F9" s="42" t="inlineStr">
-        <is>
-          <t>01</t>
-        </is>
-      </c>
-      <c r="G9" s="42" t="inlineStr">
-        <is>
-          <t>01</t>
-        </is>
-      </c>
-      <c r="H9" s="42" t="inlineStr">
-        <is>
-          <t>instansi</t>
-        </is>
-      </c>
-      <c r="I9" s="43" t="inlineStr">
-        <is>
-          <t>Infaq</t>
-        </is>
-      </c>
-      <c r="J9" s="44" t="n">
-        <v>100000</v>
-      </c>
+      <c r="A9" s="42" t="n"/>
+      <c r="B9" s="42" t="n"/>
+      <c r="C9" s="42" t="n"/>
+      <c r="D9" s="42" t="n"/>
+      <c r="E9" s="42" t="n"/>
+      <c r="F9" s="42" t="n"/>
+      <c r="G9" s="42" t="n"/>
+      <c r="H9" s="42" t="n"/>
+      <c r="I9" s="43" t="n"/>
+      <c r="J9" s="44" t="n"/>
       <c r="K9" s="10" t="n"/>
       <c r="L9" s="45" t="n"/>
       <c r="N9" s="23" t="inlineStr">
@@ -1336,52 +1264,16 @@
       <c r="S9" s="25" t="n"/>
     </row>
     <row r="10" ht="15" customHeight="1" s="16">
-      <c r="A10" s="42" t="n">
-        <v>5</v>
-      </c>
-      <c r="B10" s="42" t="inlineStr">
-        <is>
-          <t>2026-03-11</t>
-        </is>
-      </c>
-      <c r="C10" s="42" t="inlineStr">
-        <is>
-          <t>20:42</t>
-        </is>
-      </c>
-      <c r="D10" s="42" t="inlineStr">
-        <is>
-          <t>Ahmad Yusuf</t>
-        </is>
-      </c>
-      <c r="E10" s="42" t="inlineStr">
-        <is>
-          <t>Tipar Lor</t>
-        </is>
-      </c>
-      <c r="F10" s="42" t="inlineStr">
-        <is>
-          <t>01</t>
-        </is>
-      </c>
-      <c r="G10" s="42" t="inlineStr">
-        <is>
-          <t>02</t>
-        </is>
-      </c>
-      <c r="H10" s="42" t="inlineStr">
-        <is>
-          <t>perorangan</t>
-        </is>
-      </c>
-      <c r="I10" s="43" t="inlineStr">
-        <is>
-          <t>Zakat Maal</t>
-        </is>
-      </c>
-      <c r="J10" s="44" t="n">
-        <v>100000</v>
-      </c>
+      <c r="A10" s="42" t="n"/>
+      <c r="B10" s="42" t="n"/>
+      <c r="C10" s="42" t="n"/>
+      <c r="D10" s="42" t="n"/>
+      <c r="E10" s="42" t="n"/>
+      <c r="F10" s="42" t="n"/>
+      <c r="G10" s="42" t="n"/>
+      <c r="H10" s="42" t="n"/>
+      <c r="I10" s="43" t="n"/>
+      <c r="J10" s="44" t="n"/>
       <c r="K10" s="10" t="n"/>
       <c r="L10" s="45" t="n"/>
       <c r="N10" s="26" t="n"/>
@@ -1392,52 +1284,16 @@
       <c r="S10" s="28" t="n"/>
     </row>
     <row r="11" ht="15" customHeight="1" s="16">
-      <c r="A11" s="42" t="n">
-        <v>6</v>
-      </c>
-      <c r="B11" s="42" t="inlineStr">
-        <is>
-          <t>2026-03-10</t>
-        </is>
-      </c>
-      <c r="C11" s="42" t="inlineStr">
-        <is>
-          <t>19:29</t>
-        </is>
-      </c>
-      <c r="D11" s="42" t="inlineStr">
-        <is>
-          <t>Budi Umar</t>
-        </is>
-      </c>
-      <c r="E11" s="42" t="inlineStr">
-        <is>
-          <t>Tipar Kidul</t>
-        </is>
-      </c>
-      <c r="F11" s="42" t="inlineStr">
-        <is>
-          <t>01</t>
-        </is>
-      </c>
-      <c r="G11" s="42" t="inlineStr">
-        <is>
-          <t>02</t>
-        </is>
-      </c>
-      <c r="H11" s="42" t="inlineStr">
-        <is>
-          <t>perorangan</t>
-        </is>
-      </c>
-      <c r="I11" s="43" t="inlineStr">
-        <is>
-          <t>Shodaqoh</t>
-        </is>
-      </c>
-      <c r="J11" s="44" t="n">
-        <v>20000</v>
-      </c>
+      <c r="A11" s="42" t="n"/>
+      <c r="B11" s="42" t="n"/>
+      <c r="C11" s="42" t="n"/>
+      <c r="D11" s="42" t="n"/>
+      <c r="E11" s="42" t="n"/>
+      <c r="F11" s="42" t="n"/>
+      <c r="G11" s="42" t="n"/>
+      <c r="H11" s="42" t="n"/>
+      <c r="I11" s="43" t="n"/>
+      <c r="J11" s="44" t="n"/>
       <c r="K11" s="10" t="n"/>
       <c r="L11" s="45" t="n"/>
       <c r="N11" s="29" t="inlineStr">
@@ -1455,52 +1311,16 @@
       <c r="S11" s="25" t="n"/>
     </row>
     <row r="12" ht="15" customHeight="1" s="16">
-      <c r="A12" s="42" t="n">
-        <v>7</v>
-      </c>
-      <c r="B12" s="42" t="inlineStr">
-        <is>
-          <t>2026-03-05</t>
-        </is>
-      </c>
-      <c r="C12" s="42" t="inlineStr">
-        <is>
-          <t>17:44</t>
-        </is>
-      </c>
-      <c r="D12" s="42" t="inlineStr">
-        <is>
-          <t>Karim Gilang</t>
-        </is>
-      </c>
-      <c r="E12" s="42" t="inlineStr">
-        <is>
-          <t>Tipar Lor</t>
-        </is>
-      </c>
-      <c r="F12" s="42" t="inlineStr">
-        <is>
-          <t>01</t>
-        </is>
-      </c>
-      <c r="G12" s="42" t="inlineStr">
-        <is>
-          <t>02</t>
-        </is>
-      </c>
-      <c r="H12" s="42" t="inlineStr">
-        <is>
-          <t>perorangan</t>
-        </is>
-      </c>
-      <c r="I12" s="43" t="inlineStr">
-        <is>
-          <t>Infaq</t>
-        </is>
-      </c>
-      <c r="J12" s="44" t="n">
-        <v>50000</v>
-      </c>
+      <c r="A12" s="42" t="n"/>
+      <c r="B12" s="42" t="n"/>
+      <c r="C12" s="42" t="n"/>
+      <c r="D12" s="42" t="n"/>
+      <c r="E12" s="42" t="n"/>
+      <c r="F12" s="42" t="n"/>
+      <c r="G12" s="42" t="n"/>
+      <c r="H12" s="42" t="n"/>
+      <c r="I12" s="43" t="n"/>
+      <c r="J12" s="44" t="n"/>
       <c r="K12" s="10" t="n"/>
       <c r="L12" s="45" t="n"/>
       <c r="N12" s="40" t="n"/>
@@ -1511,52 +1331,16 @@
       <c r="S12" s="28" t="n"/>
     </row>
     <row r="13" ht="15" customHeight="1" s="16">
-      <c r="A13" s="42" t="n">
-        <v>8</v>
-      </c>
-      <c r="B13" s="42" t="inlineStr">
-        <is>
-          <t>2026-03-13</t>
-        </is>
-      </c>
-      <c r="C13" s="42" t="inlineStr">
-        <is>
-          <t>20:52</t>
-        </is>
-      </c>
-      <c r="D13" s="42" t="inlineStr">
-        <is>
-          <t>Naufal Indra</t>
-        </is>
-      </c>
-      <c r="E13" s="42" t="inlineStr">
-        <is>
-          <t>Tipar Lor</t>
-        </is>
-      </c>
-      <c r="F13" s="42" t="inlineStr">
-        <is>
-          <t>01</t>
-        </is>
-      </c>
-      <c r="G13" s="42" t="inlineStr">
-        <is>
-          <t>02</t>
-        </is>
-      </c>
-      <c r="H13" s="42" t="inlineStr">
-        <is>
-          <t>instansi</t>
-        </is>
-      </c>
-      <c r="I13" s="43" t="inlineStr">
-        <is>
-          <t>Infaq</t>
-        </is>
-      </c>
-      <c r="J13" s="44" t="n">
-        <v>20000</v>
-      </c>
+      <c r="A13" s="42" t="n"/>
+      <c r="B13" s="42" t="n"/>
+      <c r="C13" s="42" t="n"/>
+      <c r="D13" s="42" t="n"/>
+      <c r="E13" s="42" t="n"/>
+      <c r="F13" s="42" t="n"/>
+      <c r="G13" s="42" t="n"/>
+      <c r="H13" s="42" t="n"/>
+      <c r="I13" s="43" t="n"/>
+      <c r="J13" s="44" t="n"/>
       <c r="K13" s="10" t="n"/>
       <c r="L13" s="45" t="n"/>
       <c r="N13" s="29" t="inlineStr">
@@ -1574,52 +1358,16 @@
       <c r="S13" s="25" t="n"/>
     </row>
     <row r="14" ht="15" customHeight="1" s="16">
-      <c r="A14" s="42" t="n">
-        <v>9</v>
-      </c>
-      <c r="B14" s="42" t="inlineStr">
-        <is>
-          <t>2026-03-07</t>
-        </is>
-      </c>
-      <c r="C14" s="42" t="inlineStr">
-        <is>
-          <t>18:41</t>
-        </is>
-      </c>
-      <c r="D14" s="42" t="inlineStr">
-        <is>
-          <t>Ahmad Slamet</t>
-        </is>
-      </c>
-      <c r="E14" s="42" t="inlineStr">
-        <is>
-          <t>Ajibarang Kulon</t>
-        </is>
-      </c>
-      <c r="F14" s="42" t="inlineStr">
-        <is>
-          <t>01</t>
-        </is>
-      </c>
-      <c r="G14" s="42" t="inlineStr">
-        <is>
-          <t>03</t>
-        </is>
-      </c>
-      <c r="H14" s="42" t="inlineStr">
-        <is>
-          <t>perorangan</t>
-        </is>
-      </c>
-      <c r="I14" s="43" t="inlineStr">
-        <is>
-          <t>Shodaqoh</t>
-        </is>
-      </c>
-      <c r="J14" s="44" t="n">
-        <v>10000</v>
-      </c>
+      <c r="A14" s="42" t="n"/>
+      <c r="B14" s="42" t="n"/>
+      <c r="C14" s="42" t="n"/>
+      <c r="D14" s="42" t="n"/>
+      <c r="E14" s="42" t="n"/>
+      <c r="F14" s="42" t="n"/>
+      <c r="G14" s="42" t="n"/>
+      <c r="H14" s="42" t="n"/>
+      <c r="I14" s="43" t="n"/>
+      <c r="J14" s="44" t="n"/>
       <c r="K14" s="10" t="n"/>
       <c r="L14" s="45" t="n"/>
       <c r="N14" s="40" t="n"/>
@@ -1630,52 +1378,16 @@
       <c r="S14" s="28" t="n"/>
     </row>
     <row r="15" ht="15" customHeight="1" s="16">
-      <c r="A15" s="42" t="n">
-        <v>10</v>
-      </c>
-      <c r="B15" s="42" t="inlineStr">
-        <is>
-          <t>2026-03-13</t>
-        </is>
-      </c>
-      <c r="C15" s="42" t="inlineStr">
-        <is>
-          <t>21:45</t>
-        </is>
-      </c>
-      <c r="D15" s="42" t="inlineStr">
-        <is>
-          <t>Fajar Karim</t>
-        </is>
-      </c>
-      <c r="E15" s="42" t="inlineStr">
-        <is>
-          <t>Ajibarang Wetan</t>
-        </is>
-      </c>
-      <c r="F15" s="42" t="inlineStr">
-        <is>
-          <t>01</t>
-        </is>
-      </c>
-      <c r="G15" s="42" t="inlineStr">
-        <is>
-          <t>03</t>
-        </is>
-      </c>
-      <c r="H15" s="42" t="inlineStr">
-        <is>
-          <t>instansi</t>
-        </is>
-      </c>
-      <c r="I15" s="43" t="inlineStr">
-        <is>
-          <t>Shodaqoh</t>
-        </is>
-      </c>
-      <c r="J15" s="44" t="n">
-        <v>20000</v>
-      </c>
+      <c r="A15" s="42" t="n"/>
+      <c r="B15" s="42" t="n"/>
+      <c r="C15" s="42" t="n"/>
+      <c r="D15" s="42" t="n"/>
+      <c r="E15" s="42" t="n"/>
+      <c r="F15" s="42" t="n"/>
+      <c r="G15" s="42" t="n"/>
+      <c r="H15" s="42" t="n"/>
+      <c r="I15" s="43" t="n"/>
+      <c r="J15" s="44" t="n"/>
       <c r="K15" s="10" t="n"/>
       <c r="L15" s="45" t="n"/>
       <c r="N15" s="29" t="inlineStr">
@@ -1693,52 +1405,16 @@
       <c r="S15" s="25" t="n"/>
     </row>
     <row r="16" ht="15" customHeight="1" s="16">
-      <c r="A16" s="42" t="n">
-        <v>11</v>
-      </c>
-      <c r="B16" s="42" t="inlineStr">
-        <is>
-          <t>2026-03-11</t>
-        </is>
-      </c>
-      <c r="C16" s="42" t="inlineStr">
-        <is>
-          <t>18:34</t>
-        </is>
-      </c>
-      <c r="D16" s="42" t="inlineStr">
-        <is>
-          <t>Joko Taufik</t>
-        </is>
-      </c>
-      <c r="E16" s="42" t="inlineStr">
-        <is>
-          <t>Tipar Kidul</t>
-        </is>
-      </c>
-      <c r="F16" s="42" t="inlineStr">
-        <is>
-          <t>01</t>
-        </is>
-      </c>
-      <c r="G16" s="42" t="inlineStr">
-        <is>
-          <t>03</t>
-        </is>
-      </c>
-      <c r="H16" s="42" t="inlineStr">
-        <is>
-          <t>instansi</t>
-        </is>
-      </c>
-      <c r="I16" s="43" t="inlineStr">
-        <is>
-          <t>Infaq</t>
-        </is>
-      </c>
-      <c r="J16" s="44" t="n">
-        <v>50000</v>
-      </c>
+      <c r="A16" s="42" t="n"/>
+      <c r="B16" s="42" t="n"/>
+      <c r="C16" s="42" t="n"/>
+      <c r="D16" s="42" t="n"/>
+      <c r="E16" s="42" t="n"/>
+      <c r="F16" s="42" t="n"/>
+      <c r="G16" s="42" t="n"/>
+      <c r="H16" s="42" t="n"/>
+      <c r="I16" s="43" t="n"/>
+      <c r="J16" s="44" t="n"/>
       <c r="K16" s="10" t="n"/>
       <c r="L16" s="45" t="n"/>
       <c r="N16" s="40" t="n"/>
@@ -1749,52 +1425,16 @@
       <c r="S16" s="28" t="n"/>
     </row>
     <row r="17" ht="15" customHeight="1" s="16">
-      <c r="A17" s="42" t="n">
-        <v>12</v>
-      </c>
-      <c r="B17" s="42" t="inlineStr">
-        <is>
-          <t>2026-03-06</t>
-        </is>
-      </c>
-      <c r="C17" s="42" t="inlineStr">
-        <is>
-          <t>20:56</t>
-        </is>
-      </c>
-      <c r="D17" s="42" t="inlineStr">
-        <is>
-          <t>Rizki Lukman</t>
-        </is>
-      </c>
-      <c r="E17" s="42" t="inlineStr">
-        <is>
-          <t>Ajibarang Wetan</t>
-        </is>
-      </c>
-      <c r="F17" s="42" t="inlineStr">
-        <is>
-          <t>01</t>
-        </is>
-      </c>
-      <c r="G17" s="42" t="inlineStr">
-        <is>
-          <t>03</t>
-        </is>
-      </c>
-      <c r="H17" s="42" t="inlineStr">
-        <is>
-          <t>instansi</t>
-        </is>
-      </c>
-      <c r="I17" s="43" t="inlineStr">
-        <is>
-          <t>Shodaqoh</t>
-        </is>
-      </c>
-      <c r="J17" s="44" t="n">
-        <v>100000</v>
-      </c>
+      <c r="A17" s="42" t="n"/>
+      <c r="B17" s="42" t="n"/>
+      <c r="C17" s="42" t="n"/>
+      <c r="D17" s="42" t="n"/>
+      <c r="E17" s="42" t="n"/>
+      <c r="F17" s="42" t="n"/>
+      <c r="G17" s="42" t="n"/>
+      <c r="H17" s="42" t="n"/>
+      <c r="I17" s="43" t="n"/>
+      <c r="J17" s="44" t="n"/>
       <c r="K17" s="10" t="n"/>
       <c r="L17" s="45" t="n"/>
       <c r="N17" s="29" t="inlineStr">
@@ -1812,52 +1452,16 @@
       <c r="S17" s="25" t="n"/>
     </row>
     <row r="18" ht="15" customHeight="1" s="16">
-      <c r="A18" s="42" t="n">
-        <v>13</v>
-      </c>
-      <c r="B18" s="42" t="inlineStr">
-        <is>
-          <t>2026-03-09</t>
-        </is>
-      </c>
-      <c r="C18" s="42" t="inlineStr">
-        <is>
-          <t>20:54</t>
-        </is>
-      </c>
-      <c r="D18" s="42" t="inlineStr">
-        <is>
-          <t>Fajar Ahmad</t>
-        </is>
-      </c>
-      <c r="E18" s="42" t="inlineStr">
-        <is>
-          <t>Tipar Lor</t>
-        </is>
-      </c>
-      <c r="F18" s="42" t="inlineStr">
-        <is>
-          <t>02</t>
-        </is>
-      </c>
-      <c r="G18" s="42" t="inlineStr">
-        <is>
-          <t>01</t>
-        </is>
-      </c>
-      <c r="H18" s="42" t="inlineStr">
-        <is>
-          <t>instansi</t>
-        </is>
-      </c>
-      <c r="I18" s="43" t="inlineStr">
-        <is>
-          <t>Shodaqoh</t>
-        </is>
-      </c>
-      <c r="J18" s="44" t="n">
-        <v>100000</v>
-      </c>
+      <c r="A18" s="42" t="n"/>
+      <c r="B18" s="42" t="n"/>
+      <c r="C18" s="42" t="n"/>
+      <c r="D18" s="42" t="n"/>
+      <c r="E18" s="42" t="n"/>
+      <c r="F18" s="42" t="n"/>
+      <c r="G18" s="42" t="n"/>
+      <c r="H18" s="42" t="n"/>
+      <c r="I18" s="43" t="n"/>
+      <c r="J18" s="44" t="n"/>
       <c r="K18" s="10" t="n"/>
       <c r="L18" s="45" t="n"/>
       <c r="N18" s="40" t="n"/>
@@ -1868,52 +1472,16 @@
       <c r="S18" s="28" t="n"/>
     </row>
     <row r="19" ht="15" customHeight="1" s="16">
-      <c r="A19" s="42" t="n">
-        <v>14</v>
-      </c>
-      <c r="B19" s="42" t="inlineStr">
-        <is>
-          <t>2026-03-11</t>
-        </is>
-      </c>
-      <c r="C19" s="42" t="inlineStr">
-        <is>
-          <t>17:50</t>
-        </is>
-      </c>
-      <c r="D19" s="42" t="inlineStr">
-        <is>
-          <t>Fajar Budi</t>
-        </is>
-      </c>
-      <c r="E19" s="42" t="inlineStr">
-        <is>
-          <t>Tipar Kidul</t>
-        </is>
-      </c>
-      <c r="F19" s="42" t="inlineStr">
-        <is>
-          <t>02</t>
-        </is>
-      </c>
-      <c r="G19" s="42" t="inlineStr">
-        <is>
-          <t>01</t>
-        </is>
-      </c>
-      <c r="H19" s="42" t="inlineStr">
-        <is>
-          <t>instansi</t>
-        </is>
-      </c>
-      <c r="I19" s="43" t="inlineStr">
-        <is>
-          <t>Shodaqoh</t>
-        </is>
-      </c>
-      <c r="J19" s="44" t="n">
-        <v>100000</v>
-      </c>
+      <c r="A19" s="42" t="n"/>
+      <c r="B19" s="42" t="n"/>
+      <c r="C19" s="42" t="n"/>
+      <c r="D19" s="42" t="n"/>
+      <c r="E19" s="42" t="n"/>
+      <c r="F19" s="42" t="n"/>
+      <c r="G19" s="42" t="n"/>
+      <c r="H19" s="42" t="n"/>
+      <c r="I19" s="43" t="n"/>
+      <c r="J19" s="44" t="n"/>
       <c r="K19" s="10" t="n"/>
       <c r="L19" s="45" t="n"/>
       <c r="N19" s="29" t="inlineStr">
@@ -1931,52 +1499,16 @@
       <c r="S19" s="25" t="n"/>
     </row>
     <row r="20" ht="15" customHeight="1" s="16">
-      <c r="A20" s="42" t="n">
-        <v>15</v>
-      </c>
-      <c r="B20" s="42" t="inlineStr">
-        <is>
-          <t>2026-03-11</t>
-        </is>
-      </c>
-      <c r="C20" s="42" t="inlineStr">
-        <is>
-          <t>17:43</t>
-        </is>
-      </c>
-      <c r="D20" s="42" t="inlineStr">
-        <is>
-          <t>Hadi Rizki</t>
-        </is>
-      </c>
-      <c r="E20" s="42" t="inlineStr">
-        <is>
-          <t>Ajibarang Wetan</t>
-        </is>
-      </c>
-      <c r="F20" s="42" t="inlineStr">
-        <is>
-          <t>02</t>
-        </is>
-      </c>
-      <c r="G20" s="42" t="inlineStr">
-        <is>
-          <t>01</t>
-        </is>
-      </c>
-      <c r="H20" s="42" t="inlineStr">
-        <is>
-          <t>instansi</t>
-        </is>
-      </c>
-      <c r="I20" s="43" t="inlineStr">
-        <is>
-          <t>Shodaqoh</t>
-        </is>
-      </c>
-      <c r="J20" s="44" t="n">
-        <v>50000</v>
-      </c>
+      <c r="A20" s="42" t="n"/>
+      <c r="B20" s="42" t="n"/>
+      <c r="C20" s="42" t="n"/>
+      <c r="D20" s="42" t="n"/>
+      <c r="E20" s="42" t="n"/>
+      <c r="F20" s="42" t="n"/>
+      <c r="G20" s="42" t="n"/>
+      <c r="H20" s="42" t="n"/>
+      <c r="I20" s="43" t="n"/>
+      <c r="J20" s="44" t="n"/>
       <c r="K20" s="10" t="n"/>
       <c r="L20" s="45" t="n"/>
       <c r="N20" s="40" t="n"/>
@@ -1987,52 +1519,16 @@
       <c r="S20" s="28" t="n"/>
     </row>
     <row r="21" ht="15" customHeight="1" s="16">
-      <c r="A21" s="42" t="n">
-        <v>16</v>
-      </c>
-      <c r="B21" s="42" t="inlineStr">
-        <is>
-          <t>2026-03-13</t>
-        </is>
-      </c>
-      <c r="C21" s="42" t="inlineStr">
-        <is>
-          <t>17:11</t>
-        </is>
-      </c>
-      <c r="D21" s="42" t="inlineStr">
-        <is>
-          <t>Joko Lukman</t>
-        </is>
-      </c>
-      <c r="E21" s="42" t="inlineStr">
-        <is>
-          <t>Tipar Lor</t>
-        </is>
-      </c>
-      <c r="F21" s="42" t="inlineStr">
-        <is>
-          <t>02</t>
-        </is>
-      </c>
-      <c r="G21" s="42" t="inlineStr">
-        <is>
-          <t>01</t>
-        </is>
-      </c>
-      <c r="H21" s="42" t="inlineStr">
-        <is>
-          <t>perorangan</t>
-        </is>
-      </c>
-      <c r="I21" s="43" t="inlineStr">
-        <is>
-          <t>Infaq</t>
-        </is>
-      </c>
-      <c r="J21" s="44" t="n">
-        <v>10000</v>
-      </c>
+      <c r="A21" s="42" t="n"/>
+      <c r="B21" s="42" t="n"/>
+      <c r="C21" s="42" t="n"/>
+      <c r="D21" s="42" t="n"/>
+      <c r="E21" s="42" t="n"/>
+      <c r="F21" s="42" t="n"/>
+      <c r="G21" s="42" t="n"/>
+      <c r="H21" s="42" t="n"/>
+      <c r="I21" s="43" t="n"/>
+      <c r="J21" s="44" t="n"/>
       <c r="K21" s="10" t="n"/>
       <c r="L21" s="45" t="n"/>
       <c r="N21" s="29" t="inlineStr">
@@ -2050,52 +1546,16 @@
       <c r="S21" s="25" t="n"/>
     </row>
     <row r="22" ht="15" customHeight="1" s="16">
-      <c r="A22" s="42" t="n">
-        <v>17</v>
-      </c>
-      <c r="B22" s="42" t="inlineStr">
-        <is>
-          <t>2026-03-13</t>
-        </is>
-      </c>
-      <c r="C22" s="42" t="inlineStr">
-        <is>
-          <t>17:57</t>
-        </is>
-      </c>
-      <c r="D22" s="42" t="inlineStr">
-        <is>
-          <t>Slamet Naufal</t>
-        </is>
-      </c>
-      <c r="E22" s="42" t="inlineStr">
-        <is>
-          <t>Ajibarang Wetan</t>
-        </is>
-      </c>
-      <c r="F22" s="42" t="inlineStr">
-        <is>
-          <t>02</t>
-        </is>
-      </c>
-      <c r="G22" s="42" t="inlineStr">
-        <is>
-          <t>01</t>
-        </is>
-      </c>
-      <c r="H22" s="42" t="inlineStr">
-        <is>
-          <t>perorangan</t>
-        </is>
-      </c>
-      <c r="I22" s="43" t="inlineStr">
-        <is>
-          <t>Infaq</t>
-        </is>
-      </c>
-      <c r="J22" s="44" t="n">
-        <v>10000</v>
-      </c>
+      <c r="A22" s="42" t="n"/>
+      <c r="B22" s="42" t="n"/>
+      <c r="C22" s="42" t="n"/>
+      <c r="D22" s="42" t="n"/>
+      <c r="E22" s="42" t="n"/>
+      <c r="F22" s="42" t="n"/>
+      <c r="G22" s="42" t="n"/>
+      <c r="H22" s="42" t="n"/>
+      <c r="I22" s="43" t="n"/>
+      <c r="J22" s="44" t="n"/>
       <c r="K22" s="10" t="n"/>
       <c r="L22" s="45" t="n"/>
       <c r="N22" s="40" t="n"/>
@@ -2106,3202 +1566,898 @@
       <c r="S22" s="28" t="n"/>
     </row>
     <row r="23" ht="15" customHeight="1" s="16">
-      <c r="A23" s="42" t="n">
-        <v>18</v>
-      </c>
-      <c r="B23" s="42" t="inlineStr">
-        <is>
-          <t>2026-03-10</t>
-        </is>
-      </c>
-      <c r="C23" s="42" t="inlineStr">
-        <is>
-          <t>20:25</t>
-        </is>
-      </c>
-      <c r="D23" s="42" t="inlineStr">
-        <is>
-          <t>Ahmad Slamet</t>
-        </is>
-      </c>
-      <c r="E23" s="42" t="inlineStr">
-        <is>
-          <t>Tipar Kidul</t>
-        </is>
-      </c>
-      <c r="F23" s="42" t="inlineStr">
-        <is>
-          <t>02</t>
-        </is>
-      </c>
-      <c r="G23" s="42" t="inlineStr">
-        <is>
-          <t>02</t>
-        </is>
-      </c>
-      <c r="H23" s="42" t="inlineStr">
-        <is>
-          <t>perorangan</t>
-        </is>
-      </c>
-      <c r="I23" s="43" t="inlineStr">
-        <is>
-          <t>Shodaqoh</t>
-        </is>
-      </c>
-      <c r="J23" s="44" t="n">
-        <v>20000</v>
-      </c>
+      <c r="A23" s="42" t="n"/>
+      <c r="B23" s="42" t="n"/>
+      <c r="C23" s="42" t="n"/>
+      <c r="D23" s="42" t="n"/>
+      <c r="E23" s="42" t="n"/>
+      <c r="F23" s="42" t="n"/>
+      <c r="G23" s="42" t="n"/>
+      <c r="H23" s="42" t="n"/>
+      <c r="I23" s="43" t="n"/>
+      <c r="J23" s="44" t="n"/>
       <c r="K23" s="10" t="n"/>
       <c r="L23" s="45" t="n"/>
     </row>
     <row r="24" ht="15" customHeight="1" s="16">
-      <c r="A24" s="42" t="n">
-        <v>19</v>
-      </c>
-      <c r="B24" s="42" t="inlineStr">
-        <is>
-          <t>2026-03-06</t>
-        </is>
-      </c>
-      <c r="C24" s="42" t="inlineStr">
-        <is>
-          <t>20:47</t>
-        </is>
-      </c>
-      <c r="D24" s="42" t="inlineStr">
-        <is>
-          <t>Hadi Indra</t>
-        </is>
-      </c>
-      <c r="E24" s="42" t="inlineStr">
-        <is>
-          <t>Tipar Lor</t>
-        </is>
-      </c>
-      <c r="F24" s="42" t="inlineStr">
-        <is>
-          <t>02</t>
-        </is>
-      </c>
-      <c r="G24" s="42" t="inlineStr">
-        <is>
-          <t>02</t>
-        </is>
-      </c>
-      <c r="H24" s="42" t="inlineStr">
-        <is>
-          <t>perorangan</t>
-        </is>
-      </c>
-      <c r="I24" s="43" t="inlineStr">
-        <is>
-          <t>Infaq</t>
-        </is>
-      </c>
-      <c r="J24" s="44" t="n">
-        <v>50000</v>
-      </c>
+      <c r="A24" s="42" t="n"/>
+      <c r="B24" s="42" t="n"/>
+      <c r="C24" s="42" t="n"/>
+      <c r="D24" s="42" t="n"/>
+      <c r="E24" s="42" t="n"/>
+      <c r="F24" s="42" t="n"/>
+      <c r="G24" s="42" t="n"/>
+      <c r="H24" s="42" t="n"/>
+      <c r="I24" s="43" t="n"/>
+      <c r="J24" s="44" t="n"/>
       <c r="K24" s="10" t="n"/>
       <c r="L24" s="45" t="n"/>
     </row>
     <row r="25" ht="15" customHeight="1" s="16">
-      <c r="A25" s="42" t="n">
-        <v>20</v>
-      </c>
-      <c r="B25" s="42" t="inlineStr">
-        <is>
-          <t>2026-03-07</t>
-        </is>
-      </c>
-      <c r="C25" s="42" t="inlineStr">
-        <is>
-          <t>19:34</t>
-        </is>
-      </c>
-      <c r="D25" s="42" t="inlineStr">
-        <is>
-          <t>Karim Umar</t>
-        </is>
-      </c>
-      <c r="E25" s="42" t="inlineStr">
-        <is>
-          <t>Ajibarang Kulon</t>
-        </is>
-      </c>
-      <c r="F25" s="42" t="inlineStr">
-        <is>
-          <t>02</t>
-        </is>
-      </c>
-      <c r="G25" s="42" t="inlineStr">
-        <is>
-          <t>02</t>
-        </is>
-      </c>
-      <c r="H25" s="42" t="inlineStr">
-        <is>
-          <t>instansi</t>
-        </is>
-      </c>
-      <c r="I25" s="43" t="inlineStr">
-        <is>
-          <t>Shodaqoh</t>
-        </is>
-      </c>
-      <c r="J25" s="44" t="n">
-        <v>200000</v>
-      </c>
+      <c r="A25" s="42" t="n"/>
+      <c r="B25" s="42" t="n"/>
+      <c r="C25" s="42" t="n"/>
+      <c r="D25" s="42" t="n"/>
+      <c r="E25" s="42" t="n"/>
+      <c r="F25" s="42" t="n"/>
+      <c r="G25" s="42" t="n"/>
+      <c r="H25" s="42" t="n"/>
+      <c r="I25" s="43" t="n"/>
+      <c r="J25" s="44" t="n"/>
       <c r="K25" s="10" t="n"/>
       <c r="L25" s="45" t="n"/>
     </row>
     <row r="26" ht="15" customHeight="1" s="16">
-      <c r="A26" s="42" t="n">
-        <v>21</v>
-      </c>
-      <c r="B26" s="42" t="inlineStr">
-        <is>
-          <t>2026-03-13</t>
-        </is>
-      </c>
-      <c r="C26" s="42" t="inlineStr">
-        <is>
-          <t>20:13</t>
-        </is>
-      </c>
-      <c r="D26" s="42" t="inlineStr">
-        <is>
-          <t>Rizki Yusuf</t>
-        </is>
-      </c>
-      <c r="E26" s="42" t="inlineStr">
-        <is>
-          <t>Ajibarang Kulon</t>
-        </is>
-      </c>
-      <c r="F26" s="42" t="inlineStr">
-        <is>
-          <t>02</t>
-        </is>
-      </c>
-      <c r="G26" s="42" t="inlineStr">
-        <is>
-          <t>02</t>
-        </is>
-      </c>
-      <c r="H26" s="42" t="inlineStr">
-        <is>
-          <t>perorangan</t>
-        </is>
-      </c>
-      <c r="I26" s="43" t="inlineStr">
-        <is>
-          <t>Zakat Maal</t>
-        </is>
-      </c>
-      <c r="J26" s="44" t="n">
-        <v>200000</v>
-      </c>
+      <c r="A26" s="42" t="n"/>
+      <c r="B26" s="42" t="n"/>
+      <c r="C26" s="42" t="n"/>
+      <c r="D26" s="42" t="n"/>
+      <c r="E26" s="42" t="n"/>
+      <c r="F26" s="42" t="n"/>
+      <c r="G26" s="42" t="n"/>
+      <c r="H26" s="42" t="n"/>
+      <c r="I26" s="43" t="n"/>
+      <c r="J26" s="44" t="n"/>
       <c r="K26" s="10" t="n"/>
       <c r="L26" s="45" t="n"/>
     </row>
     <row r="27" ht="15" customHeight="1" s="16">
-      <c r="A27" s="42" t="n">
-        <v>22</v>
-      </c>
-      <c r="B27" s="42" t="inlineStr">
-        <is>
-          <t>2026-03-08</t>
-        </is>
-      </c>
-      <c r="C27" s="42" t="inlineStr">
-        <is>
-          <t>20:10</t>
-        </is>
-      </c>
-      <c r="D27" s="42" t="inlineStr">
-        <is>
-          <t>Slamet Karim</t>
-        </is>
-      </c>
-      <c r="E27" s="42" t="inlineStr">
-        <is>
-          <t>Tipar Kidul</t>
-        </is>
-      </c>
-      <c r="F27" s="42" t="inlineStr">
-        <is>
-          <t>02</t>
-        </is>
-      </c>
-      <c r="G27" s="42" t="inlineStr">
-        <is>
-          <t>02</t>
-        </is>
-      </c>
-      <c r="H27" s="42" t="inlineStr">
-        <is>
-          <t>perorangan</t>
-        </is>
-      </c>
-      <c r="I27" s="43" t="inlineStr">
-        <is>
-          <t>Zakat Maal</t>
-        </is>
-      </c>
-      <c r="J27" s="44" t="n">
-        <v>10000</v>
-      </c>
+      <c r="A27" s="42" t="n"/>
+      <c r="B27" s="42" t="n"/>
+      <c r="C27" s="42" t="n"/>
+      <c r="D27" s="42" t="n"/>
+      <c r="E27" s="42" t="n"/>
+      <c r="F27" s="42" t="n"/>
+      <c r="G27" s="42" t="n"/>
+      <c r="H27" s="42" t="n"/>
+      <c r="I27" s="43" t="n"/>
+      <c r="J27" s="44" t="n"/>
       <c r="K27" s="10" t="n"/>
       <c r="L27" s="45" t="n"/>
     </row>
     <row r="28" ht="15" customHeight="1" s="16">
-      <c r="A28" s="42" t="n">
-        <v>23</v>
-      </c>
-      <c r="B28" s="42" t="inlineStr">
-        <is>
-          <t>2026-03-03</t>
-        </is>
-      </c>
-      <c r="C28" s="42" t="inlineStr">
-        <is>
-          <t>19:25</t>
-        </is>
-      </c>
-      <c r="D28" s="42" t="inlineStr">
-        <is>
-          <t>Ahmad Hadi</t>
-        </is>
-      </c>
-      <c r="E28" s="42" t="inlineStr">
-        <is>
-          <t>Tipar Kidul</t>
-        </is>
-      </c>
-      <c r="F28" s="42" t="inlineStr">
-        <is>
-          <t>02</t>
-        </is>
-      </c>
-      <c r="G28" s="42" t="inlineStr">
-        <is>
-          <t>03</t>
-        </is>
-      </c>
-      <c r="H28" s="42" t="inlineStr">
-        <is>
-          <t>perorangan</t>
-        </is>
-      </c>
-      <c r="I28" s="43" t="inlineStr">
-        <is>
-          <t>Shodaqoh</t>
-        </is>
-      </c>
-      <c r="J28" s="44" t="n">
-        <v>10000</v>
-      </c>
+      <c r="A28" s="42" t="n"/>
+      <c r="B28" s="42" t="n"/>
+      <c r="C28" s="42" t="n"/>
+      <c r="D28" s="42" t="n"/>
+      <c r="E28" s="42" t="n"/>
+      <c r="F28" s="42" t="n"/>
+      <c r="G28" s="42" t="n"/>
+      <c r="H28" s="42" t="n"/>
+      <c r="I28" s="43" t="n"/>
+      <c r="J28" s="44" t="n"/>
       <c r="K28" s="10" t="n"/>
       <c r="L28" s="45" t="n"/>
     </row>
     <row r="29" ht="15" customHeight="1" s="16">
-      <c r="A29" s="42" t="n">
-        <v>24</v>
-      </c>
-      <c r="B29" s="42" t="inlineStr">
-        <is>
-          <t>2026-03-08</t>
-        </is>
-      </c>
-      <c r="C29" s="42" t="inlineStr">
-        <is>
-          <t>21:18</t>
-        </is>
-      </c>
-      <c r="D29" s="42" t="inlineStr">
-        <is>
-          <t>Ahmad Omar</t>
-        </is>
-      </c>
-      <c r="E29" s="42" t="inlineStr">
-        <is>
-          <t>Tipar Lor</t>
-        </is>
-      </c>
-      <c r="F29" s="42" t="inlineStr">
-        <is>
-          <t>02</t>
-        </is>
-      </c>
-      <c r="G29" s="42" t="inlineStr">
-        <is>
-          <t>03</t>
-        </is>
-      </c>
-      <c r="H29" s="42" t="inlineStr">
-        <is>
-          <t>perorangan</t>
-        </is>
-      </c>
-      <c r="I29" s="42" t="inlineStr">
-        <is>
-          <t>Zakat Maal</t>
-        </is>
-      </c>
-      <c r="J29" s="6" t="n">
-        <v>100000</v>
-      </c>
+      <c r="A29" s="42" t="n"/>
+      <c r="B29" s="42" t="n"/>
+      <c r="C29" s="42" t="n"/>
+      <c r="D29" s="42" t="n"/>
+      <c r="E29" s="42" t="n"/>
+      <c r="F29" s="42" t="n"/>
+      <c r="G29" s="42" t="n"/>
+      <c r="H29" s="42" t="n"/>
+      <c r="I29" s="42" t="n"/>
+      <c r="J29" s="6" t="n"/>
       <c r="K29" s="10" t="n"/>
       <c r="L29" s="45" t="n"/>
     </row>
     <row r="30" ht="15" customHeight="1" s="16">
-      <c r="A30" s="42" t="n">
-        <v>25</v>
-      </c>
-      <c r="B30" s="42" t="inlineStr">
-        <is>
-          <t>2026-03-07</t>
-        </is>
-      </c>
-      <c r="C30" s="42" t="inlineStr">
-        <is>
-          <t>20:22</t>
-        </is>
-      </c>
-      <c r="D30" s="42" t="inlineStr">
-        <is>
-          <t>Budi Budi</t>
-        </is>
-      </c>
-      <c r="E30" s="42" t="inlineStr">
-        <is>
-          <t>Tipar Kidul</t>
-        </is>
-      </c>
-      <c r="F30" s="42" t="inlineStr">
-        <is>
-          <t>02</t>
-        </is>
-      </c>
-      <c r="G30" s="42" t="inlineStr">
-        <is>
-          <t>03</t>
-        </is>
-      </c>
-      <c r="H30" s="42" t="inlineStr">
-        <is>
-          <t>perorangan</t>
-        </is>
-      </c>
-      <c r="I30" s="42" t="inlineStr">
-        <is>
-          <t>Shodaqoh</t>
-        </is>
-      </c>
-      <c r="J30" s="6" t="n">
-        <v>50000</v>
-      </c>
+      <c r="A30" s="42" t="n"/>
+      <c r="B30" s="42" t="n"/>
+      <c r="C30" s="42" t="n"/>
+      <c r="D30" s="42" t="n"/>
+      <c r="E30" s="42" t="n"/>
+      <c r="F30" s="42" t="n"/>
+      <c r="G30" s="42" t="n"/>
+      <c r="H30" s="42" t="n"/>
+      <c r="I30" s="42" t="n"/>
+      <c r="J30" s="6" t="n"/>
       <c r="K30" s="10" t="n"/>
       <c r="L30" s="45" t="n"/>
     </row>
     <row r="31" ht="15" customHeight="1" s="16">
-      <c r="A31" s="42" t="n">
-        <v>26</v>
-      </c>
-      <c r="B31" s="42" t="inlineStr">
-        <is>
-          <t>2026-03-11</t>
-        </is>
-      </c>
-      <c r="C31" s="42" t="inlineStr">
-        <is>
-          <t>18:28</t>
-        </is>
-      </c>
-      <c r="D31" s="42" t="inlineStr">
-        <is>
-          <t>Cahyo Slamet</t>
-        </is>
-      </c>
-      <c r="E31" s="42" t="inlineStr">
-        <is>
-          <t>Ajibarang Wetan</t>
-        </is>
-      </c>
-      <c r="F31" s="42" t="inlineStr">
-        <is>
-          <t>02</t>
-        </is>
-      </c>
-      <c r="G31" s="42" t="inlineStr">
-        <is>
-          <t>03</t>
-        </is>
-      </c>
-      <c r="H31" s="42" t="inlineStr">
-        <is>
-          <t>instansi</t>
-        </is>
-      </c>
-      <c r="I31" s="43" t="inlineStr">
-        <is>
-          <t>Zakat Maal</t>
-        </is>
-      </c>
-      <c r="J31" s="44" t="n">
-        <v>10000</v>
-      </c>
+      <c r="A31" s="42" t="n"/>
+      <c r="B31" s="42" t="n"/>
+      <c r="C31" s="42" t="n"/>
+      <c r="D31" s="42" t="n"/>
+      <c r="E31" s="42" t="n"/>
+      <c r="F31" s="42" t="n"/>
+      <c r="G31" s="42" t="n"/>
+      <c r="H31" s="42" t="n"/>
+      <c r="I31" s="43" t="n"/>
+      <c r="J31" s="44" t="n"/>
       <c r="K31" s="10" t="n"/>
       <c r="L31" s="45" t="n"/>
     </row>
     <row r="32" ht="15" customHeight="1" s="16">
-      <c r="A32" s="42" t="n">
-        <v>27</v>
-      </c>
-      <c r="B32" s="42" t="inlineStr">
-        <is>
-          <t>2026-03-12</t>
-        </is>
-      </c>
-      <c r="C32" s="42" t="inlineStr">
-        <is>
-          <t>20:40</t>
-        </is>
-      </c>
-      <c r="D32" s="42" t="inlineStr">
-        <is>
-          <t>Lukman Gilang</t>
-        </is>
-      </c>
-      <c r="E32" s="42" t="inlineStr">
-        <is>
-          <t>Ajibarang Wetan</t>
-        </is>
-      </c>
-      <c r="F32" s="42" t="inlineStr">
-        <is>
-          <t>02</t>
-        </is>
-      </c>
-      <c r="G32" s="42" t="inlineStr">
-        <is>
-          <t>03</t>
-        </is>
-      </c>
-      <c r="H32" s="42" t="inlineStr">
-        <is>
-          <t>instansi</t>
-        </is>
-      </c>
-      <c r="I32" s="43" t="inlineStr">
-        <is>
-          <t>Infaq</t>
-        </is>
-      </c>
-      <c r="J32" s="44" t="n">
-        <v>50000</v>
-      </c>
+      <c r="A32" s="42" t="n"/>
+      <c r="B32" s="42" t="n"/>
+      <c r="C32" s="42" t="n"/>
+      <c r="D32" s="42" t="n"/>
+      <c r="E32" s="42" t="n"/>
+      <c r="F32" s="42" t="n"/>
+      <c r="G32" s="42" t="n"/>
+      <c r="H32" s="42" t="n"/>
+      <c r="I32" s="43" t="n"/>
+      <c r="J32" s="44" t="n"/>
       <c r="K32" s="10" t="n"/>
       <c r="L32" s="45" t="n"/>
     </row>
     <row r="33" ht="15" customHeight="1" s="16">
-      <c r="A33" s="42" t="n">
-        <v>28</v>
-      </c>
-      <c r="B33" s="42" t="inlineStr">
-        <is>
-          <t>2026-03-06</t>
-        </is>
-      </c>
-      <c r="C33" s="42" t="inlineStr">
-        <is>
-          <t>17:22</t>
-        </is>
-      </c>
-      <c r="D33" s="42" t="inlineStr">
-        <is>
-          <t>Naufal Omar</t>
-        </is>
-      </c>
-      <c r="E33" s="42" t="inlineStr">
-        <is>
-          <t>Tipar Lor</t>
-        </is>
-      </c>
-      <c r="F33" s="42" t="inlineStr">
-        <is>
-          <t>02</t>
-        </is>
-      </c>
-      <c r="G33" s="42" t="inlineStr">
-        <is>
-          <t>03</t>
-        </is>
-      </c>
-      <c r="H33" s="42" t="inlineStr">
-        <is>
-          <t>instansi</t>
-        </is>
-      </c>
-      <c r="I33" s="43" t="inlineStr">
-        <is>
-          <t>Shodaqoh</t>
-        </is>
-      </c>
-      <c r="J33" s="44" t="n">
-        <v>20000</v>
-      </c>
+      <c r="A33" s="42" t="n"/>
+      <c r="B33" s="42" t="n"/>
+      <c r="C33" s="42" t="n"/>
+      <c r="D33" s="42" t="n"/>
+      <c r="E33" s="42" t="n"/>
+      <c r="F33" s="42" t="n"/>
+      <c r="G33" s="42" t="n"/>
+      <c r="H33" s="42" t="n"/>
+      <c r="I33" s="43" t="n"/>
+      <c r="J33" s="44" t="n"/>
       <c r="K33" s="10" t="n"/>
       <c r="L33" s="45" t="n"/>
     </row>
     <row r="34" ht="15" customHeight="1" s="16">
-      <c r="A34" s="42" t="n">
-        <v>29</v>
-      </c>
-      <c r="B34" s="42" t="inlineStr">
-        <is>
-          <t>2026-03-05</t>
-        </is>
-      </c>
-      <c r="C34" s="42" t="inlineStr">
-        <is>
-          <t>21:38</t>
-        </is>
-      </c>
-      <c r="D34" s="42" t="inlineStr">
-        <is>
-          <t>Umar Maulana</t>
-        </is>
-      </c>
-      <c r="E34" s="42" t="inlineStr">
-        <is>
-          <t>Tipar Kidul</t>
-        </is>
-      </c>
-      <c r="F34" s="42" t="inlineStr">
-        <is>
-          <t>02</t>
-        </is>
-      </c>
-      <c r="G34" s="42" t="inlineStr">
-        <is>
-          <t>03</t>
-        </is>
-      </c>
-      <c r="H34" s="42" t="inlineStr">
-        <is>
-          <t>perorangan</t>
-        </is>
-      </c>
-      <c r="I34" s="43" t="inlineStr">
-        <is>
-          <t>Shodaqoh</t>
-        </is>
-      </c>
-      <c r="J34" s="44" t="n">
-        <v>100000</v>
-      </c>
+      <c r="A34" s="42" t="n"/>
+      <c r="B34" s="42" t="n"/>
+      <c r="C34" s="42" t="n"/>
+      <c r="D34" s="42" t="n"/>
+      <c r="E34" s="42" t="n"/>
+      <c r="F34" s="42" t="n"/>
+      <c r="G34" s="42" t="n"/>
+      <c r="H34" s="42" t="n"/>
+      <c r="I34" s="43" t="n"/>
+      <c r="J34" s="44" t="n"/>
       <c r="K34" s="10" t="n"/>
       <c r="L34" s="45" t="n"/>
     </row>
     <row r="35" ht="15" customHeight="1" s="16">
-      <c r="A35" s="42" t="n">
-        <v>30</v>
-      </c>
-      <c r="B35" s="42" t="inlineStr">
-        <is>
-          <t>2026-03-05</t>
-        </is>
-      </c>
-      <c r="C35" s="42" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="D35" s="42" t="inlineStr">
-        <is>
-          <t>Budi Karim</t>
-        </is>
-      </c>
-      <c r="E35" s="42" t="inlineStr">
-        <is>
-          <t>Ajibarang Wetan</t>
-        </is>
-      </c>
-      <c r="F35" s="42" t="inlineStr">
-        <is>
-          <t>03</t>
-        </is>
-      </c>
-      <c r="G35" s="42" t="inlineStr">
-        <is>
-          <t>01</t>
-        </is>
-      </c>
-      <c r="H35" s="42" t="inlineStr">
-        <is>
-          <t>instansi</t>
-        </is>
-      </c>
-      <c r="I35" s="43" t="inlineStr">
-        <is>
-          <t>Infaq</t>
-        </is>
-      </c>
-      <c r="J35" s="44" t="n">
-        <v>10000</v>
-      </c>
+      <c r="A35" s="42" t="n"/>
+      <c r="B35" s="42" t="n"/>
+      <c r="C35" s="42" t="n"/>
+      <c r="D35" s="42" t="n"/>
+      <c r="E35" s="42" t="n"/>
+      <c r="F35" s="42" t="n"/>
+      <c r="G35" s="42" t="n"/>
+      <c r="H35" s="42" t="n"/>
+      <c r="I35" s="43" t="n"/>
+      <c r="J35" s="44" t="n"/>
       <c r="K35" s="10" t="n"/>
       <c r="L35" s="45" t="n"/>
     </row>
     <row r="36" ht="15" customHeight="1" s="16">
-      <c r="A36" s="42" t="n">
-        <v>31</v>
-      </c>
-      <c r="B36" s="42" t="inlineStr">
-        <is>
-          <t>2026-03-05</t>
-        </is>
-      </c>
-      <c r="C36" s="42" t="inlineStr">
-        <is>
-          <t>18:26</t>
-        </is>
-      </c>
-      <c r="D36" s="42" t="inlineStr">
-        <is>
-          <t>Eko Yusuf</t>
-        </is>
-      </c>
-      <c r="E36" s="42" t="inlineStr">
-        <is>
-          <t>Tipar Kidul</t>
-        </is>
-      </c>
-      <c r="F36" s="42" t="inlineStr">
-        <is>
-          <t>03</t>
-        </is>
-      </c>
-      <c r="G36" s="42" t="inlineStr">
-        <is>
-          <t>01</t>
-        </is>
-      </c>
-      <c r="H36" s="42" t="inlineStr">
-        <is>
-          <t>instansi</t>
-        </is>
-      </c>
-      <c r="I36" s="43" t="inlineStr">
-        <is>
-          <t>Shodaqoh</t>
-        </is>
-      </c>
-      <c r="J36" s="44" t="n">
-        <v>100000</v>
-      </c>
+      <c r="A36" s="42" t="n"/>
+      <c r="B36" s="42" t="n"/>
+      <c r="C36" s="42" t="n"/>
+      <c r="D36" s="42" t="n"/>
+      <c r="E36" s="42" t="n"/>
+      <c r="F36" s="42" t="n"/>
+      <c r="G36" s="42" t="n"/>
+      <c r="H36" s="42" t="n"/>
+      <c r="I36" s="43" t="n"/>
+      <c r="J36" s="44" t="n"/>
       <c r="K36" s="10" t="n"/>
       <c r="L36" s="45" t="n"/>
     </row>
     <row r="37" ht="15" customHeight="1" s="16">
-      <c r="A37" s="42" t="n">
-        <v>32</v>
-      </c>
-      <c r="B37" s="42" t="inlineStr">
-        <is>
-          <t>2026-03-07</t>
-        </is>
-      </c>
-      <c r="C37" s="42" t="inlineStr">
-        <is>
-          <t>18:47</t>
-        </is>
-      </c>
-      <c r="D37" s="42" t="inlineStr">
-        <is>
-          <t>Fajar Eko</t>
-        </is>
-      </c>
-      <c r="E37" s="42" t="inlineStr">
-        <is>
-          <t>Tipar Lor</t>
-        </is>
-      </c>
-      <c r="F37" s="42" t="inlineStr">
-        <is>
-          <t>03</t>
-        </is>
-      </c>
-      <c r="G37" s="42" t="inlineStr">
-        <is>
-          <t>01</t>
-        </is>
-      </c>
-      <c r="H37" s="42" t="inlineStr">
-        <is>
-          <t>instansi</t>
-        </is>
-      </c>
-      <c r="I37" s="43" t="inlineStr">
-        <is>
-          <t>Zakat Maal</t>
-        </is>
-      </c>
-      <c r="J37" s="44" t="n">
-        <v>200000</v>
-      </c>
+      <c r="A37" s="42" t="n"/>
+      <c r="B37" s="42" t="n"/>
+      <c r="C37" s="42" t="n"/>
+      <c r="D37" s="42" t="n"/>
+      <c r="E37" s="42" t="n"/>
+      <c r="F37" s="42" t="n"/>
+      <c r="G37" s="42" t="n"/>
+      <c r="H37" s="42" t="n"/>
+      <c r="I37" s="43" t="n"/>
+      <c r="J37" s="44" t="n"/>
       <c r="K37" s="10" t="n"/>
       <c r="L37" s="45" t="n"/>
     </row>
     <row r="38" ht="15" customHeight="1" s="16">
-      <c r="A38" s="42" t="n">
-        <v>33</v>
-      </c>
-      <c r="B38" s="42" t="inlineStr">
-        <is>
-          <t>2026-03-12</t>
-        </is>
-      </c>
-      <c r="C38" s="42" t="inlineStr">
-        <is>
-          <t>19:14</t>
-        </is>
-      </c>
-      <c r="D38" s="42" t="inlineStr">
-        <is>
-          <t>Gilang Maulana</t>
-        </is>
-      </c>
-      <c r="E38" s="42" t="inlineStr">
-        <is>
-          <t>Tipar Kidul</t>
-        </is>
-      </c>
-      <c r="F38" s="42" t="inlineStr">
-        <is>
-          <t>03</t>
-        </is>
-      </c>
-      <c r="G38" s="42" t="inlineStr">
-        <is>
-          <t>01</t>
-        </is>
-      </c>
-      <c r="H38" s="42" t="inlineStr">
-        <is>
-          <t>perorangan</t>
-        </is>
-      </c>
-      <c r="I38" s="43" t="inlineStr">
-        <is>
-          <t>Shodaqoh</t>
-        </is>
-      </c>
-      <c r="J38" s="44" t="n">
-        <v>200000</v>
-      </c>
+      <c r="A38" s="42" t="n"/>
+      <c r="B38" s="42" t="n"/>
+      <c r="C38" s="42" t="n"/>
+      <c r="D38" s="42" t="n"/>
+      <c r="E38" s="42" t="n"/>
+      <c r="F38" s="42" t="n"/>
+      <c r="G38" s="42" t="n"/>
+      <c r="H38" s="42" t="n"/>
+      <c r="I38" s="43" t="n"/>
+      <c r="J38" s="44" t="n"/>
       <c r="K38" s="10" t="n"/>
       <c r="L38" s="45" t="n"/>
     </row>
     <row r="39" ht="15" customHeight="1" s="16">
-      <c r="A39" s="42" t="n">
-        <v>34</v>
-      </c>
-      <c r="B39" s="42" t="inlineStr">
-        <is>
-          <t>2026-03-04</t>
-        </is>
-      </c>
-      <c r="C39" s="42" t="inlineStr">
-        <is>
-          <t>18:26</t>
-        </is>
-      </c>
-      <c r="D39" s="42" t="inlineStr">
-        <is>
-          <t>Slamet Karim</t>
-        </is>
-      </c>
-      <c r="E39" s="42" t="inlineStr">
-        <is>
-          <t>Ajibarang Kulon</t>
-        </is>
-      </c>
-      <c r="F39" s="42" t="inlineStr">
-        <is>
-          <t>03</t>
-        </is>
-      </c>
-      <c r="G39" s="42" t="inlineStr">
-        <is>
-          <t>01</t>
-        </is>
-      </c>
-      <c r="H39" s="42" t="inlineStr">
-        <is>
-          <t>instansi</t>
-        </is>
-      </c>
-      <c r="I39" s="43" t="inlineStr">
-        <is>
-          <t>Zakat Maal</t>
-        </is>
-      </c>
-      <c r="J39" s="44" t="n">
-        <v>200000</v>
-      </c>
+      <c r="A39" s="42" t="n"/>
+      <c r="B39" s="42" t="n"/>
+      <c r="C39" s="42" t="n"/>
+      <c r="D39" s="42" t="n"/>
+      <c r="E39" s="42" t="n"/>
+      <c r="F39" s="42" t="n"/>
+      <c r="G39" s="42" t="n"/>
+      <c r="H39" s="42" t="n"/>
+      <c r="I39" s="43" t="n"/>
+      <c r="J39" s="44" t="n"/>
       <c r="K39" s="10" t="n"/>
       <c r="L39" s="45" t="n"/>
     </row>
     <row r="40" ht="15" customHeight="1" s="16">
-      <c r="A40" s="42" t="n">
-        <v>35</v>
-      </c>
-      <c r="B40" s="42" t="inlineStr">
-        <is>
-          <t>2026-03-07</t>
-        </is>
-      </c>
-      <c r="C40" s="42" t="inlineStr">
-        <is>
-          <t>21:37</t>
-        </is>
-      </c>
-      <c r="D40" s="42" t="inlineStr">
-        <is>
-          <t>Cahyo Budi</t>
-        </is>
-      </c>
-      <c r="E40" s="42" t="inlineStr">
-        <is>
-          <t>Tipar Lor</t>
-        </is>
-      </c>
-      <c r="F40" s="42" t="inlineStr">
-        <is>
-          <t>03</t>
-        </is>
-      </c>
-      <c r="G40" s="42" t="inlineStr">
-        <is>
-          <t>02</t>
-        </is>
-      </c>
-      <c r="H40" s="42" t="inlineStr">
-        <is>
-          <t>instansi</t>
-        </is>
-      </c>
-      <c r="I40" s="43" t="inlineStr">
-        <is>
-          <t>Zakat Maal</t>
-        </is>
-      </c>
-      <c r="J40" s="44" t="n">
-        <v>10000</v>
-      </c>
+      <c r="A40" s="42" t="n"/>
+      <c r="B40" s="42" t="n"/>
+      <c r="C40" s="42" t="n"/>
+      <c r="D40" s="42" t="n"/>
+      <c r="E40" s="42" t="n"/>
+      <c r="F40" s="42" t="n"/>
+      <c r="G40" s="42" t="n"/>
+      <c r="H40" s="42" t="n"/>
+      <c r="I40" s="43" t="n"/>
+      <c r="J40" s="44" t="n"/>
       <c r="K40" s="10" t="n"/>
       <c r="L40" s="45" t="n"/>
     </row>
     <row r="41" ht="15" customHeight="1" s="16">
-      <c r="A41" s="42" t="n">
-        <v>36</v>
-      </c>
-      <c r="B41" s="42" t="inlineStr">
-        <is>
-          <t>2026-03-11</t>
-        </is>
-      </c>
-      <c r="C41" s="42" t="inlineStr">
-        <is>
-          <t>21:44</t>
-        </is>
-      </c>
-      <c r="D41" s="42" t="inlineStr">
-        <is>
-          <t>Joko Rizki</t>
-        </is>
-      </c>
-      <c r="E41" s="42" t="inlineStr">
-        <is>
-          <t>Tipar Kidul</t>
-        </is>
-      </c>
-      <c r="F41" s="42" t="inlineStr">
-        <is>
-          <t>03</t>
-        </is>
-      </c>
-      <c r="G41" s="42" t="inlineStr">
-        <is>
-          <t>02</t>
-        </is>
-      </c>
-      <c r="H41" s="42" t="inlineStr">
-        <is>
-          <t>instansi</t>
-        </is>
-      </c>
-      <c r="I41" s="43" t="inlineStr">
-        <is>
-          <t>Zakat Maal</t>
-        </is>
-      </c>
-      <c r="J41" s="44" t="n">
-        <v>200000</v>
-      </c>
+      <c r="A41" s="42" t="n"/>
+      <c r="B41" s="42" t="n"/>
+      <c r="C41" s="42" t="n"/>
+      <c r="D41" s="42" t="n"/>
+      <c r="E41" s="42" t="n"/>
+      <c r="F41" s="42" t="n"/>
+      <c r="G41" s="42" t="n"/>
+      <c r="H41" s="42" t="n"/>
+      <c r="I41" s="43" t="n"/>
+      <c r="J41" s="44" t="n"/>
       <c r="K41" s="10" t="n"/>
       <c r="L41" s="45" t="n"/>
     </row>
     <row r="42" ht="15" customHeight="1" s="16">
-      <c r="A42" s="42" t="n">
-        <v>37</v>
-      </c>
-      <c r="B42" s="42" t="inlineStr">
-        <is>
-          <t>2026-03-05</t>
-        </is>
-      </c>
-      <c r="C42" s="42" t="inlineStr">
-        <is>
-          <t>17:15</t>
-        </is>
-      </c>
-      <c r="D42" s="42" t="inlineStr">
-        <is>
-          <t>Lukman Karim</t>
-        </is>
-      </c>
-      <c r="E42" s="42" t="inlineStr">
-        <is>
-          <t>Ajibarang Wetan</t>
-        </is>
-      </c>
-      <c r="F42" s="42" t="inlineStr">
-        <is>
-          <t>03</t>
-        </is>
-      </c>
-      <c r="G42" s="42" t="inlineStr">
-        <is>
-          <t>02</t>
-        </is>
-      </c>
-      <c r="H42" s="42" t="inlineStr">
-        <is>
-          <t>instansi</t>
-        </is>
-      </c>
-      <c r="I42" s="43" t="inlineStr">
-        <is>
-          <t>Zakat Maal</t>
-        </is>
-      </c>
-      <c r="J42" s="44" t="n">
-        <v>10000</v>
-      </c>
+      <c r="A42" s="42" t="n"/>
+      <c r="B42" s="42" t="n"/>
+      <c r="C42" s="42" t="n"/>
+      <c r="D42" s="42" t="n"/>
+      <c r="E42" s="42" t="n"/>
+      <c r="F42" s="42" t="n"/>
+      <c r="G42" s="42" t="n"/>
+      <c r="H42" s="42" t="n"/>
+      <c r="I42" s="43" t="n"/>
+      <c r="J42" s="44" t="n"/>
       <c r="K42" s="10" t="n"/>
       <c r="L42" s="45" t="n"/>
     </row>
     <row r="43" ht="15" customHeight="1" s="16">
-      <c r="A43" s="42" t="n">
-        <v>38</v>
-      </c>
-      <c r="B43" s="42" t="inlineStr">
-        <is>
-          <t>2026-03-11</t>
-        </is>
-      </c>
-      <c r="C43" s="42" t="inlineStr">
-        <is>
-          <t>18:23</t>
-        </is>
-      </c>
-      <c r="D43" s="42" t="inlineStr">
-        <is>
-          <t>Maulana Eko</t>
-        </is>
-      </c>
-      <c r="E43" s="42" t="inlineStr">
-        <is>
-          <t>Tipar Lor</t>
-        </is>
-      </c>
-      <c r="F43" s="42" t="inlineStr">
-        <is>
-          <t>03</t>
-        </is>
-      </c>
-      <c r="G43" s="42" t="inlineStr">
-        <is>
-          <t>02</t>
-        </is>
-      </c>
-      <c r="H43" s="42" t="inlineStr">
-        <is>
-          <t>instansi</t>
-        </is>
-      </c>
-      <c r="I43" s="43" t="inlineStr">
-        <is>
-          <t>Infaq</t>
-        </is>
-      </c>
-      <c r="J43" s="44" t="n">
-        <v>20000</v>
-      </c>
+      <c r="A43" s="42" t="n"/>
+      <c r="B43" s="42" t="n"/>
+      <c r="C43" s="42" t="n"/>
+      <c r="D43" s="42" t="n"/>
+      <c r="E43" s="42" t="n"/>
+      <c r="F43" s="42" t="n"/>
+      <c r="G43" s="42" t="n"/>
+      <c r="H43" s="42" t="n"/>
+      <c r="I43" s="43" t="n"/>
+      <c r="J43" s="44" t="n"/>
       <c r="K43" s="10" t="n"/>
       <c r="L43" s="45" t="n"/>
     </row>
     <row r="44" ht="15" customHeight="1" s="16">
-      <c r="A44" s="42" t="n">
-        <v>39</v>
-      </c>
-      <c r="B44" s="42" t="inlineStr">
-        <is>
-          <t>2026-03-06</t>
-        </is>
-      </c>
-      <c r="C44" s="42" t="inlineStr">
-        <is>
-          <t>21:23</t>
-        </is>
-      </c>
-      <c r="D44" s="42" t="inlineStr">
-        <is>
-          <t>Naufal Taufik</t>
-        </is>
-      </c>
-      <c r="E44" s="42" t="inlineStr">
-        <is>
-          <t>Ajibarang Kulon</t>
-        </is>
-      </c>
-      <c r="F44" s="42" t="inlineStr">
-        <is>
-          <t>03</t>
-        </is>
-      </c>
-      <c r="G44" s="42" t="inlineStr">
-        <is>
-          <t>02</t>
-        </is>
-      </c>
-      <c r="H44" s="42" t="inlineStr">
-        <is>
-          <t>instansi</t>
-        </is>
-      </c>
-      <c r="I44" s="43" t="inlineStr">
-        <is>
-          <t>Zakat Maal</t>
-        </is>
-      </c>
-      <c r="J44" s="44" t="n">
-        <v>20000</v>
-      </c>
+      <c r="A44" s="42" t="n"/>
+      <c r="B44" s="42" t="n"/>
+      <c r="C44" s="42" t="n"/>
+      <c r="D44" s="42" t="n"/>
+      <c r="E44" s="42" t="n"/>
+      <c r="F44" s="42" t="n"/>
+      <c r="G44" s="42" t="n"/>
+      <c r="H44" s="42" t="n"/>
+      <c r="I44" s="43" t="n"/>
+      <c r="J44" s="44" t="n"/>
       <c r="K44" s="10" t="n"/>
       <c r="L44" s="45" t="n"/>
     </row>
     <row r="45" ht="15" customHeight="1" s="16">
-      <c r="A45" s="42" t="n">
-        <v>40</v>
-      </c>
-      <c r="B45" s="42" t="inlineStr">
-        <is>
-          <t>2026-03-06</t>
-        </is>
-      </c>
-      <c r="C45" s="42" t="inlineStr">
-        <is>
-          <t>19:48</t>
-        </is>
-      </c>
-      <c r="D45" s="42" t="inlineStr">
-        <is>
-          <t>Cahyo Dedi</t>
-        </is>
-      </c>
-      <c r="E45" s="42" t="inlineStr">
-        <is>
-          <t>Ajibarang Kulon</t>
-        </is>
-      </c>
-      <c r="F45" s="42" t="inlineStr">
-        <is>
-          <t>03</t>
-        </is>
-      </c>
-      <c r="G45" s="42" t="inlineStr">
-        <is>
-          <t>03</t>
-        </is>
-      </c>
-      <c r="H45" s="42" t="inlineStr">
-        <is>
-          <t>instansi</t>
-        </is>
-      </c>
-      <c r="I45" s="43" t="inlineStr">
-        <is>
-          <t>Zakat Maal</t>
-        </is>
-      </c>
-      <c r="J45" s="44" t="n">
-        <v>10000</v>
-      </c>
+      <c r="A45" s="42" t="n"/>
+      <c r="B45" s="42" t="n"/>
+      <c r="C45" s="42" t="n"/>
+      <c r="D45" s="42" t="n"/>
+      <c r="E45" s="42" t="n"/>
+      <c r="F45" s="42" t="n"/>
+      <c r="G45" s="42" t="n"/>
+      <c r="H45" s="42" t="n"/>
+      <c r="I45" s="43" t="n"/>
+      <c r="J45" s="44" t="n"/>
       <c r="K45" s="10" t="n"/>
       <c r="L45" s="45" t="n"/>
     </row>
     <row r="46" ht="15" customHeight="1" s="16">
-      <c r="A46" s="42" t="n">
-        <v>41</v>
-      </c>
-      <c r="B46" s="42" t="inlineStr">
-        <is>
-          <t>2026-03-05</t>
-        </is>
-      </c>
-      <c r="C46" s="42" t="inlineStr">
-        <is>
-          <t>18:28</t>
-        </is>
-      </c>
-      <c r="D46" s="42" t="inlineStr">
-        <is>
-          <t>Naufal Budi</t>
-        </is>
-      </c>
-      <c r="E46" s="42" t="inlineStr">
-        <is>
-          <t>Tipar Kidul</t>
-        </is>
-      </c>
-      <c r="F46" s="42" t="inlineStr">
-        <is>
-          <t>03</t>
-        </is>
-      </c>
-      <c r="G46" s="42" t="inlineStr">
-        <is>
-          <t>03</t>
-        </is>
-      </c>
-      <c r="H46" s="42" t="inlineStr">
-        <is>
-          <t>perorangan</t>
-        </is>
-      </c>
-      <c r="I46" s="43" t="inlineStr">
-        <is>
-          <t>Shodaqoh</t>
-        </is>
-      </c>
-      <c r="J46" s="44" t="n">
-        <v>20000</v>
-      </c>
+      <c r="A46" s="42" t="n"/>
+      <c r="B46" s="42" t="n"/>
+      <c r="C46" s="42" t="n"/>
+      <c r="D46" s="42" t="n"/>
+      <c r="E46" s="42" t="n"/>
+      <c r="F46" s="42" t="n"/>
+      <c r="G46" s="42" t="n"/>
+      <c r="H46" s="42" t="n"/>
+      <c r="I46" s="43" t="n"/>
+      <c r="J46" s="44" t="n"/>
       <c r="K46" s="10" t="n"/>
       <c r="L46" s="45" t="n"/>
     </row>
     <row r="47" ht="15" customHeight="1" s="16">
-      <c r="A47" s="42" t="n">
-        <v>42</v>
-      </c>
-      <c r="B47" s="42" t="inlineStr">
-        <is>
-          <t>2026-03-12</t>
-        </is>
-      </c>
-      <c r="C47" s="42" t="inlineStr">
-        <is>
-          <t>19:33</t>
-        </is>
-      </c>
-      <c r="D47" s="42" t="inlineStr">
-        <is>
-          <t>Umar Dedi</t>
-        </is>
-      </c>
-      <c r="E47" s="42" t="inlineStr">
-        <is>
-          <t>Tipar Lor</t>
-        </is>
-      </c>
-      <c r="F47" s="42" t="inlineStr">
-        <is>
-          <t>03</t>
-        </is>
-      </c>
-      <c r="G47" s="42" t="inlineStr">
-        <is>
-          <t>03</t>
-        </is>
-      </c>
-      <c r="H47" s="42" t="inlineStr">
-        <is>
-          <t>perorangan</t>
-        </is>
-      </c>
-      <c r="I47" s="43" t="inlineStr">
-        <is>
-          <t>Zakat Maal</t>
-        </is>
-      </c>
-      <c r="J47" s="44" t="n">
-        <v>200000</v>
-      </c>
+      <c r="A47" s="42" t="n"/>
+      <c r="B47" s="42" t="n"/>
+      <c r="C47" s="42" t="n"/>
+      <c r="D47" s="42" t="n"/>
+      <c r="E47" s="42" t="n"/>
+      <c r="F47" s="42" t="n"/>
+      <c r="G47" s="42" t="n"/>
+      <c r="H47" s="42" t="n"/>
+      <c r="I47" s="43" t="n"/>
+      <c r="J47" s="44" t="n"/>
       <c r="K47" s="10" t="n"/>
       <c r="L47" s="45" t="n"/>
     </row>
     <row r="48" ht="15" customHeight="1" s="16">
-      <c r="A48" s="42" t="n">
-        <v>43</v>
-      </c>
-      <c r="B48" s="42" t="inlineStr">
-        <is>
-          <t>2026-03-07</t>
-        </is>
-      </c>
-      <c r="C48" s="42" t="inlineStr">
-        <is>
-          <t>17:33</t>
-        </is>
-      </c>
-      <c r="D48" s="42" t="inlineStr">
-        <is>
-          <t>Ahmad Fajar</t>
-        </is>
-      </c>
-      <c r="E48" s="42" t="inlineStr">
-        <is>
-          <t>Tipar Kidul</t>
-        </is>
-      </c>
-      <c r="F48" s="42" t="inlineStr">
-        <is>
-          <t>04</t>
-        </is>
-      </c>
-      <c r="G48" s="42" t="inlineStr">
-        <is>
-          <t>01</t>
-        </is>
-      </c>
-      <c r="H48" s="42" t="inlineStr">
-        <is>
-          <t>perorangan</t>
-        </is>
-      </c>
-      <c r="I48" s="43" t="inlineStr">
-        <is>
-          <t>Zakat Maal</t>
-        </is>
-      </c>
-      <c r="J48" s="44" t="n">
-        <v>10000</v>
-      </c>
+      <c r="A48" s="42" t="n"/>
+      <c r="B48" s="42" t="n"/>
+      <c r="C48" s="42" t="n"/>
+      <c r="D48" s="42" t="n"/>
+      <c r="E48" s="42" t="n"/>
+      <c r="F48" s="42" t="n"/>
+      <c r="G48" s="42" t="n"/>
+      <c r="H48" s="42" t="n"/>
+      <c r="I48" s="43" t="n"/>
+      <c r="J48" s="44" t="n"/>
       <c r="K48" s="10" t="n"/>
       <c r="L48" s="45" t="n"/>
     </row>
     <row r="49" ht="15" customHeight="1" s="16">
-      <c r="A49" s="42" t="n">
-        <v>44</v>
-      </c>
-      <c r="B49" s="42" t="inlineStr">
-        <is>
-          <t>2026-03-05</t>
-        </is>
-      </c>
-      <c r="C49" s="42" t="inlineStr">
-        <is>
-          <t>18:55</t>
-        </is>
-      </c>
-      <c r="D49" s="42" t="inlineStr">
-        <is>
-          <t>Budi Omar</t>
-        </is>
-      </c>
-      <c r="E49" s="42" t="inlineStr">
-        <is>
-          <t>Ajibarang Wetan</t>
-        </is>
-      </c>
-      <c r="F49" s="42" t="inlineStr">
-        <is>
-          <t>04</t>
-        </is>
-      </c>
-      <c r="G49" s="42" t="inlineStr">
-        <is>
-          <t>01</t>
-        </is>
-      </c>
-      <c r="H49" s="42" t="inlineStr">
-        <is>
-          <t>perorangan</t>
-        </is>
-      </c>
-      <c r="I49" s="43" t="inlineStr">
-        <is>
-          <t>Infaq</t>
-        </is>
-      </c>
-      <c r="J49" s="44" t="n">
-        <v>100000</v>
-      </c>
+      <c r="A49" s="42" t="n"/>
+      <c r="B49" s="42" t="n"/>
+      <c r="C49" s="42" t="n"/>
+      <c r="D49" s="42" t="n"/>
+      <c r="E49" s="42" t="n"/>
+      <c r="F49" s="42" t="n"/>
+      <c r="G49" s="42" t="n"/>
+      <c r="H49" s="42" t="n"/>
+      <c r="I49" s="43" t="n"/>
+      <c r="J49" s="44" t="n"/>
       <c r="K49" s="10" t="n"/>
       <c r="L49" s="45" t="n"/>
     </row>
     <row r="50" ht="15" customHeight="1" s="16">
-      <c r="A50" s="42" t="n">
-        <v>45</v>
-      </c>
-      <c r="B50" s="42" t="inlineStr">
-        <is>
-          <t>2026-03-11</t>
-        </is>
-      </c>
-      <c r="C50" s="42" t="inlineStr">
-        <is>
-          <t>19:18</t>
-        </is>
-      </c>
-      <c r="D50" s="42" t="inlineStr">
-        <is>
-          <t>Cahyo Eko</t>
-        </is>
-      </c>
-      <c r="E50" s="42" t="inlineStr">
-        <is>
-          <t>Ajibarang Kulon</t>
-        </is>
-      </c>
-      <c r="F50" s="42" t="inlineStr">
-        <is>
-          <t>04</t>
-        </is>
-      </c>
-      <c r="G50" s="42" t="inlineStr">
-        <is>
-          <t>01</t>
-        </is>
-      </c>
-      <c r="H50" s="42" t="inlineStr">
-        <is>
-          <t>instansi</t>
-        </is>
-      </c>
-      <c r="I50" s="43" t="inlineStr">
-        <is>
-          <t>Zakat Maal</t>
-        </is>
-      </c>
-      <c r="J50" s="44" t="n">
-        <v>200000</v>
-      </c>
+      <c r="A50" s="42" t="n"/>
+      <c r="B50" s="42" t="n"/>
+      <c r="C50" s="42" t="n"/>
+      <c r="D50" s="42" t="n"/>
+      <c r="E50" s="42" t="n"/>
+      <c r="F50" s="42" t="n"/>
+      <c r="G50" s="42" t="n"/>
+      <c r="H50" s="42" t="n"/>
+      <c r="I50" s="43" t="n"/>
+      <c r="J50" s="44" t="n"/>
       <c r="K50" s="10" t="n"/>
       <c r="L50" s="45" t="n"/>
     </row>
     <row r="51" ht="15" customHeight="1" s="16">
-      <c r="A51" s="42" t="n">
-        <v>46</v>
-      </c>
-      <c r="B51" s="42" t="inlineStr">
-        <is>
-          <t>2026-03-04</t>
-        </is>
-      </c>
-      <c r="C51" s="42" t="inlineStr">
-        <is>
-          <t>20:28</t>
-        </is>
-      </c>
-      <c r="D51" s="42" t="inlineStr">
-        <is>
-          <t>Maulana Gilang</t>
-        </is>
-      </c>
-      <c r="E51" s="42" t="inlineStr">
-        <is>
-          <t>Ajibarang Kulon</t>
-        </is>
-      </c>
-      <c r="F51" s="42" t="inlineStr">
-        <is>
-          <t>04</t>
-        </is>
-      </c>
-      <c r="G51" s="42" t="inlineStr">
-        <is>
-          <t>01</t>
-        </is>
-      </c>
-      <c r="H51" s="42" t="inlineStr">
-        <is>
-          <t>instansi</t>
-        </is>
-      </c>
-      <c r="I51" s="43" t="inlineStr">
-        <is>
-          <t>Infaq</t>
-        </is>
-      </c>
-      <c r="J51" s="44" t="n">
-        <v>10000</v>
-      </c>
+      <c r="A51" s="42" t="n"/>
+      <c r="B51" s="42" t="n"/>
+      <c r="C51" s="42" t="n"/>
+      <c r="D51" s="42" t="n"/>
+      <c r="E51" s="42" t="n"/>
+      <c r="F51" s="42" t="n"/>
+      <c r="G51" s="42" t="n"/>
+      <c r="H51" s="42" t="n"/>
+      <c r="I51" s="43" t="n"/>
+      <c r="J51" s="44" t="n"/>
       <c r="K51" s="10" t="n"/>
       <c r="L51" s="45" t="n"/>
     </row>
     <row r="52" ht="15" customHeight="1" s="16">
-      <c r="A52" s="42" t="n">
-        <v>47</v>
-      </c>
-      <c r="B52" s="42" t="inlineStr">
-        <is>
-          <t>2026-03-10</t>
-        </is>
-      </c>
-      <c r="C52" s="42" t="inlineStr">
-        <is>
-          <t>20:10</t>
-        </is>
-      </c>
-      <c r="D52" s="42" t="inlineStr">
-        <is>
-          <t>Maulana Karim</t>
-        </is>
-      </c>
-      <c r="E52" s="42" t="inlineStr">
-        <is>
-          <t>Tipar Lor</t>
-        </is>
-      </c>
-      <c r="F52" s="42" t="inlineStr">
-        <is>
-          <t>04</t>
-        </is>
-      </c>
-      <c r="G52" s="42" t="inlineStr">
-        <is>
-          <t>01</t>
-        </is>
-      </c>
-      <c r="H52" s="42" t="inlineStr">
-        <is>
-          <t>perorangan</t>
-        </is>
-      </c>
-      <c r="I52" s="43" t="inlineStr">
-        <is>
-          <t>Zakat Maal</t>
-        </is>
-      </c>
-      <c r="J52" s="44" t="n">
-        <v>10000</v>
-      </c>
+      <c r="A52" s="42" t="n"/>
+      <c r="B52" s="42" t="n"/>
+      <c r="C52" s="42" t="n"/>
+      <c r="D52" s="42" t="n"/>
+      <c r="E52" s="42" t="n"/>
+      <c r="F52" s="42" t="n"/>
+      <c r="G52" s="42" t="n"/>
+      <c r="H52" s="42" t="n"/>
+      <c r="I52" s="43" t="n"/>
+      <c r="J52" s="44" t="n"/>
       <c r="K52" s="10" t="n"/>
       <c r="L52" s="45" t="n"/>
     </row>
     <row r="53" ht="15" customHeight="1" s="16">
-      <c r="A53" s="42" t="n">
-        <v>48</v>
-      </c>
-      <c r="B53" s="42" t="inlineStr">
-        <is>
-          <t>2026-03-13</t>
-        </is>
-      </c>
-      <c r="C53" s="42" t="inlineStr">
-        <is>
-          <t>20:35</t>
-        </is>
-      </c>
-      <c r="D53" s="42" t="inlineStr">
-        <is>
-          <t>Omar Karim</t>
-        </is>
-      </c>
-      <c r="E53" s="42" t="inlineStr">
-        <is>
-          <t>Tipar Lor</t>
-        </is>
-      </c>
-      <c r="F53" s="42" t="inlineStr">
-        <is>
-          <t>04</t>
-        </is>
-      </c>
-      <c r="G53" s="42" t="inlineStr">
-        <is>
-          <t>01</t>
-        </is>
-      </c>
-      <c r="H53" s="42" t="inlineStr">
-        <is>
-          <t>perorangan</t>
-        </is>
-      </c>
-      <c r="I53" s="43" t="inlineStr">
-        <is>
-          <t>Zakat Maal</t>
-        </is>
-      </c>
-      <c r="J53" s="44" t="n">
-        <v>10000</v>
-      </c>
+      <c r="A53" s="42" t="n"/>
+      <c r="B53" s="42" t="n"/>
+      <c r="C53" s="42" t="n"/>
+      <c r="D53" s="42" t="n"/>
+      <c r="E53" s="42" t="n"/>
+      <c r="F53" s="42" t="n"/>
+      <c r="G53" s="42" t="n"/>
+      <c r="H53" s="42" t="n"/>
+      <c r="I53" s="43" t="n"/>
+      <c r="J53" s="44" t="n"/>
       <c r="K53" s="10" t="n"/>
       <c r="L53" s="45" t="n"/>
     </row>
     <row r="54" ht="15" customHeight="1" s="16">
-      <c r="A54" s="42" t="n">
-        <v>49</v>
-      </c>
-      <c r="B54" s="42" t="inlineStr">
-        <is>
-          <t>2026-03-11</t>
-        </is>
-      </c>
-      <c r="C54" s="42" t="inlineStr">
-        <is>
-          <t>21:29</t>
-        </is>
-      </c>
-      <c r="D54" s="42" t="inlineStr">
-        <is>
-          <t>Taufik Lukman</t>
-        </is>
-      </c>
-      <c r="E54" s="42" t="inlineStr">
-        <is>
-          <t>Ajibarang Wetan</t>
-        </is>
-      </c>
-      <c r="F54" s="42" t="inlineStr">
-        <is>
-          <t>04</t>
-        </is>
-      </c>
-      <c r="G54" s="42" t="inlineStr">
-        <is>
-          <t>01</t>
-        </is>
-      </c>
-      <c r="H54" s="42" t="inlineStr">
-        <is>
-          <t>instansi</t>
-        </is>
-      </c>
-      <c r="I54" s="43" t="inlineStr">
-        <is>
-          <t>Infaq</t>
-        </is>
-      </c>
-      <c r="J54" s="44" t="n">
-        <v>200000</v>
-      </c>
+      <c r="A54" s="42" t="n"/>
+      <c r="B54" s="42" t="n"/>
+      <c r="C54" s="42" t="n"/>
+      <c r="D54" s="42" t="n"/>
+      <c r="E54" s="42" t="n"/>
+      <c r="F54" s="42" t="n"/>
+      <c r="G54" s="42" t="n"/>
+      <c r="H54" s="42" t="n"/>
+      <c r="I54" s="43" t="n"/>
+      <c r="J54" s="44" t="n"/>
       <c r="K54" s="10" t="n"/>
       <c r="L54" s="45" t="n"/>
     </row>
     <row r="55" ht="15" customHeight="1" s="16">
-      <c r="A55" s="42" t="n">
-        <v>50</v>
-      </c>
-      <c r="B55" s="42" t="inlineStr">
-        <is>
-          <t>2026-03-09</t>
-        </is>
-      </c>
-      <c r="C55" s="42" t="inlineStr">
-        <is>
-          <t>17:47</t>
-        </is>
-      </c>
-      <c r="D55" s="42" t="inlineStr">
-        <is>
-          <t>Umar Karim</t>
-        </is>
-      </c>
-      <c r="E55" s="42" t="inlineStr">
-        <is>
-          <t>Tipar Kidul</t>
-        </is>
-      </c>
-      <c r="F55" s="42" t="inlineStr">
-        <is>
-          <t>04</t>
-        </is>
-      </c>
-      <c r="G55" s="42" t="inlineStr">
-        <is>
-          <t>01</t>
-        </is>
-      </c>
-      <c r="H55" s="42" t="inlineStr">
-        <is>
-          <t>perorangan</t>
-        </is>
-      </c>
-      <c r="I55" s="43" t="inlineStr">
-        <is>
-          <t>Shodaqoh</t>
-        </is>
-      </c>
-      <c r="J55" s="44" t="n">
-        <v>10000</v>
-      </c>
+      <c r="A55" s="42" t="n"/>
+      <c r="B55" s="42" t="n"/>
+      <c r="C55" s="42" t="n"/>
+      <c r="D55" s="42" t="n"/>
+      <c r="E55" s="42" t="n"/>
+      <c r="F55" s="42" t="n"/>
+      <c r="G55" s="42" t="n"/>
+      <c r="H55" s="42" t="n"/>
+      <c r="I55" s="43" t="n"/>
+      <c r="J55" s="44" t="n"/>
       <c r="K55" s="10" t="n"/>
       <c r="L55" s="45" t="n"/>
     </row>
     <row r="56" ht="15" customHeight="1" s="16">
-      <c r="A56" s="42" t="n">
-        <v>51</v>
-      </c>
-      <c r="B56" s="42" t="inlineStr">
-        <is>
-          <t>2026-03-04</t>
-        </is>
-      </c>
-      <c r="C56" s="42" t="inlineStr">
-        <is>
-          <t>17:22</t>
-        </is>
-      </c>
-      <c r="D56" s="42" t="inlineStr">
-        <is>
-          <t>Cahyo Gilang</t>
-        </is>
-      </c>
-      <c r="E56" s="42" t="inlineStr">
-        <is>
-          <t>Ajibarang Wetan</t>
-        </is>
-      </c>
-      <c r="F56" s="42" t="inlineStr">
-        <is>
-          <t>04</t>
-        </is>
-      </c>
-      <c r="G56" s="42" t="inlineStr">
-        <is>
-          <t>02</t>
-        </is>
-      </c>
-      <c r="H56" s="42" t="inlineStr">
-        <is>
-          <t>perorangan</t>
-        </is>
-      </c>
-      <c r="I56" s="43" t="inlineStr">
-        <is>
-          <t>Zakat Maal</t>
-        </is>
-      </c>
-      <c r="J56" s="44" t="n">
-        <v>100000</v>
-      </c>
+      <c r="A56" s="42" t="n"/>
+      <c r="B56" s="42" t="n"/>
+      <c r="C56" s="42" t="n"/>
+      <c r="D56" s="42" t="n"/>
+      <c r="E56" s="42" t="n"/>
+      <c r="F56" s="42" t="n"/>
+      <c r="G56" s="42" t="n"/>
+      <c r="H56" s="42" t="n"/>
+      <c r="I56" s="43" t="n"/>
+      <c r="J56" s="44" t="n"/>
       <c r="K56" s="10" t="n"/>
       <c r="L56" s="45" t="n"/>
     </row>
     <row r="57" ht="15" customHeight="1" s="16">
-      <c r="A57" s="42" t="n">
-        <v>52</v>
-      </c>
-      <c r="B57" s="42" t="inlineStr">
-        <is>
-          <t>2026-03-07</t>
-        </is>
-      </c>
-      <c r="C57" s="42" t="inlineStr">
-        <is>
-          <t>20:27</t>
-        </is>
-      </c>
-      <c r="D57" s="42" t="inlineStr">
-        <is>
-          <t>Fajar Karim</t>
-        </is>
-      </c>
-      <c r="E57" s="42" t="inlineStr">
-        <is>
-          <t>Tipar Lor</t>
-        </is>
-      </c>
-      <c r="F57" s="42" t="inlineStr">
-        <is>
-          <t>04</t>
-        </is>
-      </c>
-      <c r="G57" s="42" t="inlineStr">
-        <is>
-          <t>02</t>
-        </is>
-      </c>
-      <c r="H57" s="42" t="inlineStr">
-        <is>
-          <t>perorangan</t>
-        </is>
-      </c>
-      <c r="I57" s="43" t="inlineStr">
-        <is>
-          <t>Infaq</t>
-        </is>
-      </c>
-      <c r="J57" s="44" t="n">
-        <v>50000</v>
-      </c>
+      <c r="A57" s="42" t="n"/>
+      <c r="B57" s="42" t="n"/>
+      <c r="C57" s="42" t="n"/>
+      <c r="D57" s="42" t="n"/>
+      <c r="E57" s="42" t="n"/>
+      <c r="F57" s="42" t="n"/>
+      <c r="G57" s="42" t="n"/>
+      <c r="H57" s="42" t="n"/>
+      <c r="I57" s="43" t="n"/>
+      <c r="J57" s="44" t="n"/>
       <c r="K57" s="10" t="n"/>
       <c r="L57" s="45" t="n"/>
     </row>
     <row r="58" ht="15" customHeight="1" s="16">
-      <c r="A58" s="42" t="n">
-        <v>53</v>
-      </c>
-      <c r="B58" s="42" t="inlineStr">
-        <is>
-          <t>2026-03-05</t>
-        </is>
-      </c>
-      <c r="C58" s="42" t="inlineStr">
-        <is>
-          <t>17:41</t>
-        </is>
-      </c>
-      <c r="D58" s="42" t="inlineStr">
-        <is>
-          <t>Indra Ahmad</t>
-        </is>
-      </c>
-      <c r="E58" s="42" t="inlineStr">
-        <is>
-          <t>Ajibarang Kulon</t>
-        </is>
-      </c>
-      <c r="F58" s="42" t="inlineStr">
-        <is>
-          <t>04</t>
-        </is>
-      </c>
-      <c r="G58" s="42" t="inlineStr">
-        <is>
-          <t>02</t>
-        </is>
-      </c>
-      <c r="H58" s="42" t="inlineStr">
-        <is>
-          <t>perorangan</t>
-        </is>
-      </c>
-      <c r="I58" s="43" t="inlineStr">
-        <is>
-          <t>Zakat Maal</t>
-        </is>
-      </c>
-      <c r="J58" s="44" t="n">
-        <v>100000</v>
-      </c>
+      <c r="A58" s="42" t="n"/>
+      <c r="B58" s="42" t="n"/>
+      <c r="C58" s="42" t="n"/>
+      <c r="D58" s="42" t="n"/>
+      <c r="E58" s="42" t="n"/>
+      <c r="F58" s="42" t="n"/>
+      <c r="G58" s="42" t="n"/>
+      <c r="H58" s="42" t="n"/>
+      <c r="I58" s="43" t="n"/>
+      <c r="J58" s="44" t="n"/>
       <c r="K58" s="10" t="n"/>
       <c r="L58" s="45" t="n"/>
     </row>
     <row r="59" ht="15" customHeight="1" s="16">
-      <c r="A59" s="42" t="n">
-        <v>54</v>
-      </c>
-      <c r="B59" s="42" t="inlineStr">
-        <is>
-          <t>2026-03-06</t>
-        </is>
-      </c>
-      <c r="C59" s="42" t="inlineStr">
-        <is>
-          <t>20:32</t>
-        </is>
-      </c>
-      <c r="D59" s="42" t="inlineStr">
-        <is>
-          <t>Taufik Dedi</t>
-        </is>
-      </c>
-      <c r="E59" s="42" t="inlineStr">
-        <is>
-          <t>Tipar Kidul</t>
-        </is>
-      </c>
-      <c r="F59" s="42" t="inlineStr">
-        <is>
-          <t>04</t>
-        </is>
-      </c>
-      <c r="G59" s="42" t="inlineStr">
-        <is>
-          <t>02</t>
-        </is>
-      </c>
-      <c r="H59" s="42" t="inlineStr">
-        <is>
-          <t>perorangan</t>
-        </is>
-      </c>
-      <c r="I59" s="43" t="inlineStr">
-        <is>
-          <t>Zakat Maal</t>
-        </is>
-      </c>
-      <c r="J59" s="44" t="n">
-        <v>50000</v>
-      </c>
+      <c r="A59" s="42" t="n"/>
+      <c r="B59" s="42" t="n"/>
+      <c r="C59" s="42" t="n"/>
+      <c r="D59" s="42" t="n"/>
+      <c r="E59" s="42" t="n"/>
+      <c r="F59" s="42" t="n"/>
+      <c r="G59" s="42" t="n"/>
+      <c r="H59" s="42" t="n"/>
+      <c r="I59" s="43" t="n"/>
+      <c r="J59" s="44" t="n"/>
       <c r="K59" s="10" t="n"/>
       <c r="L59" s="45" t="n"/>
     </row>
     <row r="60" ht="15" customHeight="1" s="16">
-      <c r="A60" s="42" t="n">
-        <v>55</v>
-      </c>
-      <c r="B60" s="42" t="inlineStr">
-        <is>
-          <t>2026-03-05</t>
-        </is>
-      </c>
-      <c r="C60" s="42" t="inlineStr">
-        <is>
-          <t>19:25</t>
-        </is>
-      </c>
-      <c r="D60" s="42" t="inlineStr">
-        <is>
-          <t>Budi Dedi</t>
-        </is>
-      </c>
-      <c r="E60" s="42" t="inlineStr">
-        <is>
-          <t>Ajibarang Wetan</t>
-        </is>
-      </c>
-      <c r="F60" s="42" t="inlineStr">
-        <is>
-          <t>04</t>
-        </is>
-      </c>
-      <c r="G60" s="42" t="inlineStr">
-        <is>
-          <t>03</t>
-        </is>
-      </c>
-      <c r="H60" s="42" t="inlineStr">
-        <is>
-          <t>instansi</t>
-        </is>
-      </c>
-      <c r="I60" s="43" t="inlineStr">
-        <is>
-          <t>Shodaqoh</t>
-        </is>
-      </c>
-      <c r="J60" s="44" t="n">
-        <v>100000</v>
-      </c>
+      <c r="A60" s="42" t="n"/>
+      <c r="B60" s="42" t="n"/>
+      <c r="C60" s="42" t="n"/>
+      <c r="D60" s="42" t="n"/>
+      <c r="E60" s="42" t="n"/>
+      <c r="F60" s="42" t="n"/>
+      <c r="G60" s="42" t="n"/>
+      <c r="H60" s="42" t="n"/>
+      <c r="I60" s="43" t="n"/>
+      <c r="J60" s="44" t="n"/>
       <c r="K60" s="10" t="n"/>
       <c r="L60" s="45" t="n"/>
     </row>
     <row r="61" ht="15" customHeight="1" s="16">
-      <c r="A61" s="42" t="n">
-        <v>56</v>
-      </c>
-      <c r="B61" s="42" t="inlineStr">
-        <is>
-          <t>2026-03-12</t>
-        </is>
-      </c>
-      <c r="C61" s="42" t="inlineStr">
-        <is>
-          <t>20:26</t>
-        </is>
-      </c>
-      <c r="D61" s="42" t="inlineStr">
-        <is>
-          <t>Eko Karim</t>
-        </is>
-      </c>
-      <c r="E61" s="42" t="inlineStr">
-        <is>
-          <t>Tipar Lor</t>
-        </is>
-      </c>
-      <c r="F61" s="42" t="inlineStr">
-        <is>
-          <t>04</t>
-        </is>
-      </c>
-      <c r="G61" s="42" t="inlineStr">
-        <is>
-          <t>03</t>
-        </is>
-      </c>
-      <c r="H61" s="42" t="inlineStr">
-        <is>
-          <t>perorangan</t>
-        </is>
-      </c>
-      <c r="I61" s="43" t="inlineStr">
-        <is>
-          <t>Zakat Maal</t>
-        </is>
-      </c>
-      <c r="J61" s="44" t="n">
-        <v>50000</v>
-      </c>
+      <c r="A61" s="42" t="n"/>
+      <c r="B61" s="42" t="n"/>
+      <c r="C61" s="42" t="n"/>
+      <c r="D61" s="42" t="n"/>
+      <c r="E61" s="42" t="n"/>
+      <c r="F61" s="42" t="n"/>
+      <c r="G61" s="42" t="n"/>
+      <c r="H61" s="42" t="n"/>
+      <c r="I61" s="43" t="n"/>
+      <c r="J61" s="44" t="n"/>
       <c r="K61" s="10" t="n"/>
       <c r="L61" s="45" t="n"/>
     </row>
     <row r="62" ht="15" customHeight="1" s="16">
-      <c r="A62" s="42" t="n">
-        <v>57</v>
-      </c>
-      <c r="B62" s="42" t="inlineStr">
-        <is>
-          <t>2026-03-10</t>
-        </is>
-      </c>
-      <c r="C62" s="42" t="inlineStr">
-        <is>
-          <t>21:25</t>
-        </is>
-      </c>
-      <c r="D62" s="42" t="inlineStr">
-        <is>
-          <t>Gilang Hadi</t>
-        </is>
-      </c>
-      <c r="E62" s="42" t="inlineStr">
-        <is>
-          <t>Tipar Lor</t>
-        </is>
-      </c>
-      <c r="F62" s="42" t="inlineStr">
-        <is>
-          <t>04</t>
-        </is>
-      </c>
-      <c r="G62" s="42" t="inlineStr">
-        <is>
-          <t>03</t>
-        </is>
-      </c>
-      <c r="H62" s="42" t="inlineStr">
-        <is>
-          <t>instansi</t>
-        </is>
-      </c>
-      <c r="I62" s="43" t="inlineStr">
-        <is>
-          <t>Shodaqoh</t>
-        </is>
-      </c>
-      <c r="J62" s="44" t="n">
-        <v>100000</v>
-      </c>
+      <c r="A62" s="42" t="n"/>
+      <c r="B62" s="42" t="n"/>
+      <c r="C62" s="42" t="n"/>
+      <c r="D62" s="42" t="n"/>
+      <c r="E62" s="42" t="n"/>
+      <c r="F62" s="42" t="n"/>
+      <c r="G62" s="42" t="n"/>
+      <c r="H62" s="42" t="n"/>
+      <c r="I62" s="43" t="n"/>
+      <c r="J62" s="44" t="n"/>
       <c r="K62" s="10" t="n"/>
       <c r="L62" s="45" t="n"/>
     </row>
     <row r="63" ht="15" customHeight="1" s="16">
-      <c r="A63" s="42" t="n">
-        <v>58</v>
-      </c>
-      <c r="B63" s="42" t="inlineStr">
-        <is>
-          <t>2026-03-12</t>
-        </is>
-      </c>
-      <c r="C63" s="42" t="inlineStr">
-        <is>
-          <t>17:26</t>
-        </is>
-      </c>
-      <c r="D63" s="42" t="inlineStr">
-        <is>
-          <t>Joko Karim</t>
-        </is>
-      </c>
-      <c r="E63" s="42" t="inlineStr">
-        <is>
-          <t>Tipar Lor</t>
-        </is>
-      </c>
-      <c r="F63" s="42" t="inlineStr">
-        <is>
-          <t>04</t>
-        </is>
-      </c>
-      <c r="G63" s="42" t="inlineStr">
-        <is>
-          <t>03</t>
-        </is>
-      </c>
-      <c r="H63" s="42" t="inlineStr">
-        <is>
-          <t>perorangan</t>
-        </is>
-      </c>
-      <c r="I63" s="43" t="inlineStr">
-        <is>
-          <t>Infaq</t>
-        </is>
-      </c>
-      <c r="J63" s="44" t="n">
-        <v>10000</v>
-      </c>
+      <c r="A63" s="42" t="n"/>
+      <c r="B63" s="42" t="n"/>
+      <c r="C63" s="42" t="n"/>
+      <c r="D63" s="42" t="n"/>
+      <c r="E63" s="42" t="n"/>
+      <c r="F63" s="42" t="n"/>
+      <c r="G63" s="42" t="n"/>
+      <c r="H63" s="42" t="n"/>
+      <c r="I63" s="43" t="n"/>
+      <c r="J63" s="44" t="n"/>
       <c r="K63" s="10" t="n"/>
       <c r="L63" s="45" t="n"/>
     </row>
     <row r="64" ht="15" customHeight="1" s="16">
-      <c r="A64" s="42" t="n">
-        <v>59</v>
-      </c>
-      <c r="B64" s="42" t="inlineStr">
-        <is>
-          <t>2026-03-04</t>
-        </is>
-      </c>
-      <c r="C64" s="42" t="inlineStr">
-        <is>
-          <t>19:54</t>
-        </is>
-      </c>
-      <c r="D64" s="42" t="inlineStr">
-        <is>
-          <t>Lukman Indra</t>
-        </is>
-      </c>
-      <c r="E64" s="42" t="inlineStr">
-        <is>
-          <t>Tipar Lor</t>
-        </is>
-      </c>
-      <c r="F64" s="42" t="inlineStr">
-        <is>
-          <t>04</t>
-        </is>
-      </c>
-      <c r="G64" s="42" t="inlineStr">
-        <is>
-          <t>03</t>
-        </is>
-      </c>
-      <c r="H64" s="42" t="inlineStr">
-        <is>
-          <t>instansi</t>
-        </is>
-      </c>
-      <c r="I64" s="43" t="inlineStr">
-        <is>
-          <t>Zakat Maal</t>
-        </is>
-      </c>
-      <c r="J64" s="44" t="n">
-        <v>20000</v>
-      </c>
+      <c r="A64" s="42" t="n"/>
+      <c r="B64" s="42" t="n"/>
+      <c r="C64" s="42" t="n"/>
+      <c r="D64" s="42" t="n"/>
+      <c r="E64" s="42" t="n"/>
+      <c r="F64" s="42" t="n"/>
+      <c r="G64" s="42" t="n"/>
+      <c r="H64" s="42" t="n"/>
+      <c r="I64" s="43" t="n"/>
+      <c r="J64" s="44" t="n"/>
       <c r="K64" s="10" t="n"/>
       <c r="L64" s="45" t="n"/>
     </row>
     <row r="65" ht="15" customHeight="1" s="16">
-      <c r="A65" s="42" t="n">
-        <v>60</v>
-      </c>
-      <c r="B65" s="42" t="inlineStr">
-        <is>
-          <t>2026-03-11</t>
-        </is>
-      </c>
-      <c r="C65" s="42" t="inlineStr">
-        <is>
-          <t>18:19</t>
-        </is>
-      </c>
-      <c r="D65" s="42" t="inlineStr">
-        <is>
-          <t>Maulana Naufal</t>
-        </is>
-      </c>
-      <c r="E65" s="42" t="inlineStr">
-        <is>
-          <t>Tipar Lor</t>
-        </is>
-      </c>
-      <c r="F65" s="42" t="inlineStr">
-        <is>
-          <t>04</t>
-        </is>
-      </c>
-      <c r="G65" s="42" t="inlineStr">
-        <is>
-          <t>03</t>
-        </is>
-      </c>
-      <c r="H65" s="42" t="inlineStr">
-        <is>
-          <t>instansi</t>
-        </is>
-      </c>
-      <c r="I65" s="43" t="inlineStr">
-        <is>
-          <t>Shodaqoh</t>
-        </is>
-      </c>
-      <c r="J65" s="44" t="n">
-        <v>10000</v>
-      </c>
+      <c r="A65" s="42" t="n"/>
+      <c r="B65" s="42" t="n"/>
+      <c r="C65" s="42" t="n"/>
+      <c r="D65" s="42" t="n"/>
+      <c r="E65" s="42" t="n"/>
+      <c r="F65" s="42" t="n"/>
+      <c r="G65" s="42" t="n"/>
+      <c r="H65" s="42" t="n"/>
+      <c r="I65" s="43" t="n"/>
+      <c r="J65" s="44" t="n"/>
       <c r="K65" s="10" t="n"/>
       <c r="L65" s="45" t="n"/>
     </row>
     <row r="66" ht="15" customHeight="1" s="16">
-      <c r="A66" s="42" t="n">
-        <v>61</v>
-      </c>
-      <c r="B66" s="42" t="inlineStr">
-        <is>
-          <t>2026-03-08</t>
-        </is>
-      </c>
-      <c r="C66" s="42" t="inlineStr">
-        <is>
-          <t>17:28</t>
-        </is>
-      </c>
-      <c r="D66" s="42" t="inlineStr">
-        <is>
-          <t>Naufal Taufik</t>
-        </is>
-      </c>
-      <c r="E66" s="42" t="inlineStr">
-        <is>
-          <t>Ajibarang Kulon</t>
-        </is>
-      </c>
-      <c r="F66" s="42" t="inlineStr">
-        <is>
-          <t>04</t>
-        </is>
-      </c>
-      <c r="G66" s="42" t="inlineStr">
-        <is>
-          <t>03</t>
-        </is>
-      </c>
-      <c r="H66" s="42" t="inlineStr">
-        <is>
-          <t>instansi</t>
-        </is>
-      </c>
-      <c r="I66" s="43" t="inlineStr">
-        <is>
-          <t>Zakat Maal</t>
-        </is>
-      </c>
-      <c r="J66" s="44" t="n">
-        <v>20000</v>
-      </c>
+      <c r="A66" s="42" t="n"/>
+      <c r="B66" s="42" t="n"/>
+      <c r="C66" s="42" t="n"/>
+      <c r="D66" s="42" t="n"/>
+      <c r="E66" s="42" t="n"/>
+      <c r="F66" s="42" t="n"/>
+      <c r="G66" s="42" t="n"/>
+      <c r="H66" s="42" t="n"/>
+      <c r="I66" s="43" t="n"/>
+      <c r="J66" s="44" t="n"/>
       <c r="K66" s="10" t="n"/>
       <c r="L66" s="45" t="n"/>
     </row>
     <row r="67" ht="15" customHeight="1" s="16">
-      <c r="A67" s="42" t="n">
-        <v>62</v>
-      </c>
-      <c r="B67" s="42" t="inlineStr">
-        <is>
-          <t>2026-03-10</t>
-        </is>
-      </c>
-      <c r="C67" s="42" t="inlineStr">
-        <is>
-          <t>18:55</t>
-        </is>
-      </c>
-      <c r="D67" s="42" t="inlineStr">
-        <is>
-          <t>Umar Cahyo</t>
-        </is>
-      </c>
-      <c r="E67" s="42" t="inlineStr">
-        <is>
-          <t>Ajibarang Kulon</t>
-        </is>
-      </c>
-      <c r="F67" s="42" t="inlineStr">
-        <is>
-          <t>04</t>
-        </is>
-      </c>
-      <c r="G67" s="42" t="inlineStr">
-        <is>
-          <t>03</t>
-        </is>
-      </c>
-      <c r="H67" s="42" t="inlineStr">
-        <is>
-          <t>instansi</t>
-        </is>
-      </c>
-      <c r="I67" s="43" t="inlineStr">
-        <is>
-          <t>Infaq</t>
-        </is>
-      </c>
-      <c r="J67" s="44" t="n">
-        <v>20000</v>
-      </c>
+      <c r="A67" s="42" t="n"/>
+      <c r="B67" s="42" t="n"/>
+      <c r="C67" s="42" t="n"/>
+      <c r="D67" s="42" t="n"/>
+      <c r="E67" s="42" t="n"/>
+      <c r="F67" s="42" t="n"/>
+      <c r="G67" s="42" t="n"/>
+      <c r="H67" s="42" t="n"/>
+      <c r="I67" s="43" t="n"/>
+      <c r="J67" s="44" t="n"/>
       <c r="K67" s="10" t="n"/>
       <c r="L67" s="45" t="n"/>
     </row>
     <row r="68" ht="15" customHeight="1" s="16">
-      <c r="A68" s="42" t="n">
-        <v>63</v>
-      </c>
-      <c r="B68" s="42" t="inlineStr">
-        <is>
-          <t>2026-03-05</t>
-        </is>
-      </c>
-      <c r="C68" s="42" t="inlineStr">
-        <is>
-          <t>19:19</t>
-        </is>
-      </c>
-      <c r="D68" s="42" t="inlineStr">
-        <is>
-          <t>Eko Karim</t>
-        </is>
-      </c>
-      <c r="E68" s="42" t="inlineStr">
-        <is>
-          <t>Tipar Lor</t>
-        </is>
-      </c>
-      <c r="F68" s="42" t="inlineStr">
-        <is>
-          <t>05</t>
-        </is>
-      </c>
-      <c r="G68" s="42" t="inlineStr">
-        <is>
-          <t>01</t>
-        </is>
-      </c>
-      <c r="H68" s="42" t="inlineStr">
-        <is>
-          <t>perorangan</t>
-        </is>
-      </c>
-      <c r="I68" s="43" t="inlineStr">
-        <is>
-          <t>Shodaqoh</t>
-        </is>
-      </c>
-      <c r="J68" s="44" t="n">
-        <v>50000</v>
-      </c>
+      <c r="A68" s="42" t="n"/>
+      <c r="B68" s="42" t="n"/>
+      <c r="C68" s="42" t="n"/>
+      <c r="D68" s="42" t="n"/>
+      <c r="E68" s="42" t="n"/>
+      <c r="F68" s="42" t="n"/>
+      <c r="G68" s="42" t="n"/>
+      <c r="H68" s="42" t="n"/>
+      <c r="I68" s="43" t="n"/>
+      <c r="J68" s="44" t="n"/>
       <c r="K68" s="10" t="n"/>
       <c r="L68" s="45" t="n"/>
     </row>
     <row r="69" ht="15" customHeight="1" s="16">
-      <c r="A69" s="42" t="n">
-        <v>64</v>
-      </c>
-      <c r="B69" s="42" t="inlineStr">
-        <is>
-          <t>2026-03-04</t>
-        </is>
-      </c>
-      <c r="C69" s="42" t="inlineStr">
-        <is>
-          <t>18:13</t>
-        </is>
-      </c>
-      <c r="D69" s="42" t="inlineStr">
-        <is>
-          <t>Gilang Naufal</t>
-        </is>
-      </c>
-      <c r="E69" s="42" t="inlineStr">
-        <is>
-          <t>Tipar Lor</t>
-        </is>
-      </c>
-      <c r="F69" s="42" t="inlineStr">
-        <is>
-          <t>05</t>
-        </is>
-      </c>
-      <c r="G69" s="42" t="inlineStr">
-        <is>
-          <t>01</t>
-        </is>
-      </c>
-      <c r="H69" s="42" t="inlineStr">
-        <is>
-          <t>instansi</t>
-        </is>
-      </c>
-      <c r="I69" s="43" t="inlineStr">
-        <is>
-          <t>Shodaqoh</t>
-        </is>
-      </c>
-      <c r="J69" s="44" t="n">
-        <v>200000</v>
-      </c>
+      <c r="A69" s="42" t="n"/>
+      <c r="B69" s="42" t="n"/>
+      <c r="C69" s="42" t="n"/>
+      <c r="D69" s="42" t="n"/>
+      <c r="E69" s="42" t="n"/>
+      <c r="F69" s="42" t="n"/>
+      <c r="G69" s="42" t="n"/>
+      <c r="H69" s="42" t="n"/>
+      <c r="I69" s="43" t="n"/>
+      <c r="J69" s="44" t="n"/>
       <c r="K69" s="10" t="n"/>
       <c r="L69" s="45" t="n"/>
     </row>
     <row r="70" ht="15" customHeight="1" s="16">
-      <c r="A70" s="42" t="n">
-        <v>65</v>
-      </c>
-      <c r="B70" s="42" t="inlineStr">
-        <is>
-          <t>2026-03-12</t>
-        </is>
-      </c>
-      <c r="C70" s="42" t="inlineStr">
-        <is>
-          <t>21:44</t>
-        </is>
-      </c>
-      <c r="D70" s="42" t="inlineStr">
-        <is>
-          <t>Gilang Slamet</t>
-        </is>
-      </c>
-      <c r="E70" s="42" t="inlineStr">
-        <is>
-          <t>Ajibarang Kulon</t>
-        </is>
-      </c>
-      <c r="F70" s="42" t="inlineStr">
-        <is>
-          <t>05</t>
-        </is>
-      </c>
-      <c r="G70" s="42" t="inlineStr">
-        <is>
-          <t>01</t>
-        </is>
-      </c>
-      <c r="H70" s="42" t="inlineStr">
-        <is>
-          <t>perorangan</t>
-        </is>
-      </c>
-      <c r="I70" s="43" t="inlineStr">
-        <is>
-          <t>Zakat Maal</t>
-        </is>
-      </c>
-      <c r="J70" s="44" t="n">
-        <v>100000</v>
-      </c>
+      <c r="A70" s="42" t="n"/>
+      <c r="B70" s="42" t="n"/>
+      <c r="C70" s="42" t="n"/>
+      <c r="D70" s="42" t="n"/>
+      <c r="E70" s="42" t="n"/>
+      <c r="F70" s="42" t="n"/>
+      <c r="G70" s="42" t="n"/>
+      <c r="H70" s="42" t="n"/>
+      <c r="I70" s="43" t="n"/>
+      <c r="J70" s="44" t="n"/>
       <c r="K70" s="10" t="n"/>
       <c r="L70" s="45" t="n"/>
     </row>
     <row r="71" ht="15" customHeight="1" s="16">
-      <c r="A71" s="42" t="n">
-        <v>66</v>
-      </c>
-      <c r="B71" s="42" t="inlineStr">
-        <is>
-          <t>2026-03-08</t>
-        </is>
-      </c>
-      <c r="C71" s="42" t="inlineStr">
-        <is>
-          <t>20:44</t>
-        </is>
-      </c>
-      <c r="D71" s="42" t="inlineStr">
-        <is>
-          <t>Indra Joko</t>
-        </is>
-      </c>
-      <c r="E71" s="42" t="inlineStr">
-        <is>
-          <t>Tipar Kidul</t>
-        </is>
-      </c>
-      <c r="F71" s="42" t="inlineStr">
-        <is>
-          <t>05</t>
-        </is>
-      </c>
-      <c r="G71" s="42" t="inlineStr">
-        <is>
-          <t>01</t>
-        </is>
-      </c>
-      <c r="H71" s="42" t="inlineStr">
-        <is>
-          <t>instansi</t>
-        </is>
-      </c>
-      <c r="I71" s="43" t="inlineStr">
-        <is>
-          <t>Infaq</t>
-        </is>
-      </c>
-      <c r="J71" s="44" t="n">
-        <v>50000</v>
-      </c>
+      <c r="A71" s="42" t="n"/>
+      <c r="B71" s="42" t="n"/>
+      <c r="C71" s="42" t="n"/>
+      <c r="D71" s="42" t="n"/>
+      <c r="E71" s="42" t="n"/>
+      <c r="F71" s="42" t="n"/>
+      <c r="G71" s="42" t="n"/>
+      <c r="H71" s="42" t="n"/>
+      <c r="I71" s="43" t="n"/>
+      <c r="J71" s="44" t="n"/>
       <c r="K71" s="10" t="n"/>
       <c r="L71" s="45" t="n"/>
     </row>
     <row r="72" ht="15" customHeight="1" s="16">
-      <c r="A72" s="42" t="n">
-        <v>67</v>
-      </c>
-      <c r="B72" s="42" t="inlineStr">
-        <is>
-          <t>2026-03-07</t>
-        </is>
-      </c>
-      <c r="C72" s="42" t="inlineStr">
-        <is>
-          <t>19:20</t>
-        </is>
-      </c>
-      <c r="D72" s="42" t="inlineStr">
-        <is>
-          <t>Indra Slamet</t>
-        </is>
-      </c>
-      <c r="E72" s="42" t="inlineStr">
-        <is>
-          <t>Ajibarang Wetan</t>
-        </is>
-      </c>
-      <c r="F72" s="42" t="inlineStr">
-        <is>
-          <t>05</t>
-        </is>
-      </c>
-      <c r="G72" s="42" t="inlineStr">
-        <is>
-          <t>01</t>
-        </is>
-      </c>
-      <c r="H72" s="42" t="inlineStr">
-        <is>
-          <t>instansi</t>
-        </is>
-      </c>
-      <c r="I72" s="43" t="inlineStr">
-        <is>
-          <t>Zakat Maal</t>
-        </is>
-      </c>
-      <c r="J72" s="44" t="n">
-        <v>100000</v>
-      </c>
+      <c r="A72" s="42" t="n"/>
+      <c r="B72" s="42" t="n"/>
+      <c r="C72" s="42" t="n"/>
+      <c r="D72" s="42" t="n"/>
+      <c r="E72" s="42" t="n"/>
+      <c r="F72" s="42" t="n"/>
+      <c r="G72" s="42" t="n"/>
+      <c r="H72" s="42" t="n"/>
+      <c r="I72" s="43" t="n"/>
+      <c r="J72" s="44" t="n"/>
       <c r="K72" s="10" t="n"/>
       <c r="L72" s="45" t="n"/>
     </row>
     <row r="73" ht="15" customHeight="1" s="16">
-      <c r="A73" s="42" t="n">
-        <v>68</v>
-      </c>
-      <c r="B73" s="42" t="inlineStr">
-        <is>
-          <t>2026-03-07</t>
-        </is>
-      </c>
-      <c r="C73" s="42" t="inlineStr">
-        <is>
-          <t>19:25</t>
-        </is>
-      </c>
-      <c r="D73" s="42" t="inlineStr">
-        <is>
-          <t>Joko Slamet</t>
-        </is>
-      </c>
-      <c r="E73" s="42" t="inlineStr">
-        <is>
-          <t>Tipar Kidul</t>
-        </is>
-      </c>
-      <c r="F73" s="42" t="inlineStr">
-        <is>
-          <t>05</t>
-        </is>
-      </c>
-      <c r="G73" s="42" t="inlineStr">
-        <is>
-          <t>01</t>
-        </is>
-      </c>
-      <c r="H73" s="42" t="inlineStr">
-        <is>
-          <t>perorangan</t>
-        </is>
-      </c>
-      <c r="I73" s="43" t="inlineStr">
-        <is>
-          <t>Infaq</t>
-        </is>
-      </c>
-      <c r="J73" s="44" t="n">
-        <v>100000</v>
-      </c>
+      <c r="A73" s="42" t="n"/>
+      <c r="B73" s="42" t="n"/>
+      <c r="C73" s="42" t="n"/>
+      <c r="D73" s="42" t="n"/>
+      <c r="E73" s="42" t="n"/>
+      <c r="F73" s="42" t="n"/>
+      <c r="G73" s="42" t="n"/>
+      <c r="H73" s="42" t="n"/>
+      <c r="I73" s="43" t="n"/>
+      <c r="J73" s="44" t="n"/>
       <c r="K73" s="10" t="n"/>
       <c r="L73" s="45" t="n"/>
     </row>
     <row r="74" ht="15" customHeight="1" s="16">
-      <c r="A74" s="42" t="n">
-        <v>69</v>
-      </c>
-      <c r="B74" s="42" t="inlineStr">
-        <is>
-          <t>2026-03-03</t>
-        </is>
-      </c>
-      <c r="C74" s="42" t="inlineStr">
-        <is>
-          <t>17:55</t>
-        </is>
-      </c>
-      <c r="D74" s="42" t="inlineStr">
-        <is>
-          <t>Slamet Indra</t>
-        </is>
-      </c>
-      <c r="E74" s="42" t="inlineStr">
-        <is>
-          <t>Ajibarang Wetan</t>
-        </is>
-      </c>
-      <c r="F74" s="42" t="inlineStr">
-        <is>
-          <t>05</t>
-        </is>
-      </c>
-      <c r="G74" s="42" t="inlineStr">
-        <is>
-          <t>01</t>
-        </is>
-      </c>
-      <c r="H74" s="42" t="inlineStr">
-        <is>
-          <t>instansi</t>
-        </is>
-      </c>
-      <c r="I74" s="43" t="inlineStr">
-        <is>
-          <t>Shodaqoh</t>
-        </is>
-      </c>
-      <c r="J74" s="44" t="n">
-        <v>10000</v>
-      </c>
+      <c r="A74" s="42" t="n"/>
+      <c r="B74" s="42" t="n"/>
+      <c r="C74" s="42" t="n"/>
+      <c r="D74" s="42" t="n"/>
+      <c r="E74" s="42" t="n"/>
+      <c r="F74" s="42" t="n"/>
+      <c r="G74" s="42" t="n"/>
+      <c r="H74" s="42" t="n"/>
+      <c r="I74" s="43" t="n"/>
+      <c r="J74" s="44" t="n"/>
       <c r="K74" s="10" t="n"/>
       <c r="L74" s="45" t="n"/>
     </row>
     <row r="75" ht="15" customHeight="1" s="16">
-      <c r="A75" s="42" t="n">
-        <v>70</v>
-      </c>
-      <c r="B75" s="42" t="inlineStr">
-        <is>
-          <t>2026-03-10</t>
-        </is>
-      </c>
-      <c r="C75" s="42" t="inlineStr">
-        <is>
-          <t>21:27</t>
-        </is>
-      </c>
-      <c r="D75" s="42" t="inlineStr">
-        <is>
-          <t>Slamet Maulana</t>
-        </is>
-      </c>
-      <c r="E75" s="42" t="inlineStr">
-        <is>
-          <t>Tipar Kidul</t>
-        </is>
-      </c>
-      <c r="F75" s="42" t="inlineStr">
-        <is>
-          <t>05</t>
-        </is>
-      </c>
-      <c r="G75" s="42" t="inlineStr">
-        <is>
-          <t>01</t>
-        </is>
-      </c>
-      <c r="H75" s="42" t="inlineStr">
-        <is>
-          <t>perorangan</t>
-        </is>
-      </c>
-      <c r="I75" s="43" t="inlineStr">
-        <is>
-          <t>Zakat Maal</t>
-        </is>
-      </c>
-      <c r="J75" s="44" t="n">
-        <v>20000</v>
-      </c>
+      <c r="A75" s="42" t="n"/>
+      <c r="B75" s="42" t="n"/>
+      <c r="C75" s="42" t="n"/>
+      <c r="D75" s="42" t="n"/>
+      <c r="E75" s="42" t="n"/>
+      <c r="F75" s="42" t="n"/>
+      <c r="G75" s="42" t="n"/>
+      <c r="H75" s="42" t="n"/>
+      <c r="I75" s="43" t="n"/>
+      <c r="J75" s="44" t="n"/>
       <c r="K75" s="10" t="n"/>
       <c r="L75" s="45" t="n"/>
     </row>
     <row r="76" ht="15" customHeight="1" s="16">
-      <c r="A76" s="42" t="n">
-        <v>71</v>
-      </c>
-      <c r="B76" s="42" t="inlineStr">
-        <is>
-          <t>2026-03-12</t>
-        </is>
-      </c>
-      <c r="C76" s="42" t="inlineStr">
-        <is>
-          <t>18:31</t>
-        </is>
-      </c>
-      <c r="D76" s="42" t="inlineStr">
-        <is>
-          <t>Hadi Taufik</t>
-        </is>
-      </c>
-      <c r="E76" s="42" t="inlineStr">
-        <is>
-          <t>Tipar Kidul</t>
-        </is>
-      </c>
-      <c r="F76" s="42" t="inlineStr">
-        <is>
-          <t>05</t>
-        </is>
-      </c>
-      <c r="G76" s="42" t="inlineStr">
-        <is>
-          <t>02</t>
-        </is>
-      </c>
-      <c r="H76" s="42" t="inlineStr">
-        <is>
-          <t>perorangan</t>
-        </is>
-      </c>
-      <c r="I76" s="43" t="inlineStr">
-        <is>
-          <t>Infaq</t>
-        </is>
-      </c>
-      <c r="J76" s="44" t="n">
-        <v>200000</v>
-      </c>
+      <c r="A76" s="42" t="n"/>
+      <c r="B76" s="42" t="n"/>
+      <c r="C76" s="42" t="n"/>
+      <c r="D76" s="42" t="n"/>
+      <c r="E76" s="42" t="n"/>
+      <c r="F76" s="42" t="n"/>
+      <c r="G76" s="42" t="n"/>
+      <c r="H76" s="42" t="n"/>
+      <c r="I76" s="43" t="n"/>
+      <c r="J76" s="44" t="n"/>
       <c r="K76" s="10" t="n"/>
       <c r="L76" s="45" t="n"/>
     </row>
     <row r="77" ht="15" customHeight="1" s="16">
-      <c r="A77" s="42" t="n">
-        <v>72</v>
-      </c>
-      <c r="B77" s="42" t="inlineStr">
-        <is>
-          <t>2026-03-12</t>
-        </is>
-      </c>
-      <c r="C77" s="42" t="inlineStr">
-        <is>
-          <t>17:55</t>
-        </is>
-      </c>
-      <c r="D77" s="42" t="inlineStr">
-        <is>
-          <t>Karim Fajar</t>
-        </is>
-      </c>
-      <c r="E77" s="42" t="inlineStr">
-        <is>
-          <t>Tipar Lor</t>
-        </is>
-      </c>
-      <c r="F77" s="42" t="inlineStr">
-        <is>
-          <t>05</t>
-        </is>
-      </c>
-      <c r="G77" s="42" t="inlineStr">
-        <is>
-          <t>02</t>
-        </is>
-      </c>
-      <c r="H77" s="42" t="inlineStr">
-        <is>
-          <t>instansi</t>
-        </is>
-      </c>
-      <c r="I77" s="43" t="inlineStr">
-        <is>
-          <t>Zakat Maal</t>
-        </is>
-      </c>
-      <c r="J77" s="44" t="n">
-        <v>100000</v>
-      </c>
+      <c r="A77" s="42" t="n"/>
+      <c r="B77" s="42" t="n"/>
+      <c r="C77" s="42" t="n"/>
+      <c r="D77" s="42" t="n"/>
+      <c r="E77" s="42" t="n"/>
+      <c r="F77" s="42" t="n"/>
+      <c r="G77" s="42" t="n"/>
+      <c r="H77" s="42" t="n"/>
+      <c r="I77" s="43" t="n"/>
+      <c r="J77" s="44" t="n"/>
       <c r="K77" s="10" t="n"/>
       <c r="L77" s="45" t="n"/>
     </row>
     <row r="78" ht="15" customHeight="1" s="16">
-      <c r="A78" s="42" t="n">
-        <v>73</v>
-      </c>
-      <c r="B78" s="42" t="inlineStr">
-        <is>
-          <t>2026-03-07</t>
-        </is>
-      </c>
-      <c r="C78" s="42" t="inlineStr">
-        <is>
-          <t>17:28</t>
-        </is>
-      </c>
-      <c r="D78" s="42" t="inlineStr">
-        <is>
-          <t>Naufal Maulana</t>
-        </is>
-      </c>
-      <c r="E78" s="42" t="inlineStr">
-        <is>
-          <t>Tipar Lor</t>
-        </is>
-      </c>
-      <c r="F78" s="42" t="inlineStr">
-        <is>
-          <t>05</t>
-        </is>
-      </c>
-      <c r="G78" s="42" t="inlineStr">
-        <is>
-          <t>02</t>
-        </is>
-      </c>
-      <c r="H78" s="42" t="inlineStr">
-        <is>
-          <t>instansi</t>
-        </is>
-      </c>
-      <c r="I78" s="43" t="inlineStr">
-        <is>
-          <t>Shodaqoh</t>
-        </is>
-      </c>
-      <c r="J78" s="44" t="n">
-        <v>50000</v>
-      </c>
+      <c r="A78" s="42" t="n"/>
+      <c r="B78" s="42" t="n"/>
+      <c r="C78" s="42" t="n"/>
+      <c r="D78" s="42" t="n"/>
+      <c r="E78" s="42" t="n"/>
+      <c r="F78" s="42" t="n"/>
+      <c r="G78" s="42" t="n"/>
+      <c r="H78" s="42" t="n"/>
+      <c r="I78" s="43" t="n"/>
+      <c r="J78" s="44" t="n"/>
       <c r="K78" s="10" t="n"/>
       <c r="L78" s="45" t="n"/>
     </row>
     <row r="79" ht="15" customHeight="1" s="16">
-      <c r="A79" s="42" t="n">
-        <v>74</v>
-      </c>
-      <c r="B79" s="42" t="inlineStr">
-        <is>
-          <t>2026-03-08</t>
-        </is>
-      </c>
-      <c r="C79" s="42" t="inlineStr">
-        <is>
-          <t>19:41</t>
-        </is>
-      </c>
-      <c r="D79" s="42" t="inlineStr">
-        <is>
-          <t>Yusuf Rizki</t>
-        </is>
-      </c>
-      <c r="E79" s="42" t="inlineStr">
-        <is>
-          <t>Tipar Lor</t>
-        </is>
-      </c>
-      <c r="F79" s="42" t="inlineStr">
-        <is>
-          <t>05</t>
-        </is>
-      </c>
-      <c r="G79" s="42" t="inlineStr">
-        <is>
-          <t>02</t>
-        </is>
-      </c>
-      <c r="H79" s="42" t="inlineStr">
-        <is>
-          <t>instansi</t>
-        </is>
-      </c>
-      <c r="I79" s="43" t="inlineStr">
-        <is>
-          <t>Shodaqoh</t>
-        </is>
-      </c>
-      <c r="J79" s="44" t="n">
-        <v>50000</v>
-      </c>
+      <c r="A79" s="42" t="n"/>
+      <c r="B79" s="42" t="n"/>
+      <c r="C79" s="42" t="n"/>
+      <c r="D79" s="42" t="n"/>
+      <c r="E79" s="42" t="n"/>
+      <c r="F79" s="42" t="n"/>
+      <c r="G79" s="42" t="n"/>
+      <c r="H79" s="42" t="n"/>
+      <c r="I79" s="43" t="n"/>
+      <c r="J79" s="44" t="n"/>
       <c r="K79" s="10" t="n"/>
       <c r="L79" s="45" t="n"/>
     </row>
     <row r="80" ht="15" customHeight="1" s="16">
-      <c r="A80" s="42" t="n">
-        <v>75</v>
-      </c>
-      <c r="B80" s="42" t="inlineStr">
-        <is>
-          <t>2026-03-10</t>
-        </is>
-      </c>
-      <c r="C80" s="42" t="inlineStr">
-        <is>
-          <t>18:33</t>
-        </is>
-      </c>
-      <c r="D80" s="42" t="inlineStr">
-        <is>
-          <t>Dedi Gilang</t>
-        </is>
-      </c>
-      <c r="E80" s="42" t="inlineStr">
-        <is>
-          <t>Ajibarang Kulon</t>
-        </is>
-      </c>
-      <c r="F80" s="42" t="inlineStr">
-        <is>
-          <t>05</t>
-        </is>
-      </c>
-      <c r="G80" s="42" t="inlineStr">
-        <is>
-          <t>03</t>
-        </is>
-      </c>
-      <c r="H80" s="42" t="inlineStr">
-        <is>
-          <t>perorangan</t>
-        </is>
-      </c>
-      <c r="I80" s="43" t="inlineStr">
-        <is>
-          <t>Shodaqoh</t>
-        </is>
-      </c>
-      <c r="J80" s="44" t="n">
-        <v>50000</v>
-      </c>
+      <c r="A80" s="42" t="n"/>
+      <c r="B80" s="42" t="n"/>
+      <c r="C80" s="42" t="n"/>
+      <c r="D80" s="42" t="n"/>
+      <c r="E80" s="42" t="n"/>
+      <c r="F80" s="42" t="n"/>
+      <c r="G80" s="42" t="n"/>
+      <c r="H80" s="42" t="n"/>
+      <c r="I80" s="43" t="n"/>
+      <c r="J80" s="44" t="n"/>
       <c r="K80" s="10" t="n"/>
       <c r="L80" s="45" t="n"/>
     </row>
     <row r="81" ht="15" customHeight="1" s="16">
-      <c r="A81" s="42" t="n">
-        <v>76</v>
-      </c>
-      <c r="B81" s="42" t="inlineStr">
-        <is>
-          <t>2026-03-05</t>
-        </is>
-      </c>
-      <c r="C81" s="42" t="inlineStr">
-        <is>
-          <t>18:23</t>
-        </is>
-      </c>
-      <c r="D81" s="42" t="inlineStr">
-        <is>
-          <t>Gilang Taufik</t>
-        </is>
-      </c>
-      <c r="E81" s="42" t="inlineStr">
-        <is>
-          <t>Ajibarang Wetan</t>
-        </is>
-      </c>
-      <c r="F81" s="42" t="inlineStr">
-        <is>
-          <t>05</t>
-        </is>
-      </c>
-      <c r="G81" s="42" t="inlineStr">
-        <is>
-          <t>03</t>
-        </is>
-      </c>
-      <c r="H81" s="42" t="inlineStr">
-        <is>
-          <t>instansi</t>
-        </is>
-      </c>
-      <c r="I81" s="43" t="inlineStr">
-        <is>
-          <t>Shodaqoh</t>
-        </is>
-      </c>
-      <c r="J81" s="44" t="n">
-        <v>200001</v>
-      </c>
+      <c r="A81" s="42" t="n"/>
+      <c r="B81" s="42" t="n"/>
+      <c r="C81" s="42" t="n"/>
+      <c r="D81" s="42" t="n"/>
+      <c r="E81" s="42" t="n"/>
+      <c r="F81" s="42" t="n"/>
+      <c r="G81" s="42" t="n"/>
+      <c r="H81" s="42" t="n"/>
+      <c r="I81" s="43" t="n"/>
+      <c r="J81" s="44" t="n"/>
       <c r="K81" s="10" t="n"/>
       <c r="L81" s="45" t="n"/>
     </row>
     <row r="82" ht="15" customHeight="1" s="16">
-      <c r="A82" s="42" t="n">
-        <v>77</v>
-      </c>
-      <c r="B82" s="42" t="inlineStr">
-        <is>
-          <t>2026-03-08</t>
-        </is>
-      </c>
-      <c r="C82" s="42" t="inlineStr">
-        <is>
-          <t>21:47</t>
-        </is>
-      </c>
-      <c r="D82" s="42" t="inlineStr">
-        <is>
-          <t>Hadi Slamet</t>
-        </is>
-      </c>
-      <c r="E82" s="42" t="inlineStr">
-        <is>
-          <t>Tipar Kidul</t>
-        </is>
-      </c>
-      <c r="F82" s="42" t="inlineStr">
-        <is>
-          <t>05</t>
-        </is>
-      </c>
-      <c r="G82" s="42" t="inlineStr">
-        <is>
-          <t>03</t>
-        </is>
-      </c>
-      <c r="H82" s="42" t="inlineStr">
-        <is>
-          <t>instansi</t>
-        </is>
-      </c>
-      <c r="I82" s="43" t="inlineStr">
-        <is>
-          <t>Zakat Maal</t>
-        </is>
-      </c>
-      <c r="J82" s="44" t="n">
-        <v>200000</v>
-      </c>
+      <c r="A82" s="42" t="n"/>
+      <c r="B82" s="42" t="n"/>
+      <c r="C82" s="42" t="n"/>
+      <c r="D82" s="42" t="n"/>
+      <c r="E82" s="42" t="n"/>
+      <c r="F82" s="42" t="n"/>
+      <c r="G82" s="42" t="n"/>
+      <c r="H82" s="42" t="n"/>
+      <c r="I82" s="43" t="n"/>
+      <c r="J82" s="44" t="n"/>
       <c r="K82" s="10" t="n"/>
       <c r="L82" s="45" t="n"/>
     </row>
     <row r="83" ht="15" customHeight="1" s="16">
-      <c r="A83" s="42" t="n">
-        <v>78</v>
-      </c>
-      <c r="B83" s="42" t="inlineStr">
-        <is>
-          <t>2026-03-05</t>
-        </is>
-      </c>
-      <c r="C83" s="42" t="inlineStr">
-        <is>
-          <t>20:50</t>
-        </is>
-      </c>
-      <c r="D83" s="42" t="inlineStr">
-        <is>
-          <t>Karim Yusuf</t>
-        </is>
-      </c>
-      <c r="E83" s="42" t="inlineStr">
-        <is>
-          <t>Ajibarang Wetan</t>
-        </is>
-      </c>
-      <c r="F83" s="42" t="inlineStr">
-        <is>
-          <t>05</t>
-        </is>
-      </c>
-      <c r="G83" s="42" t="inlineStr">
-        <is>
-          <t>03</t>
-        </is>
-      </c>
-      <c r="H83" s="42" t="inlineStr">
-        <is>
-          <t>instansi</t>
-        </is>
-      </c>
-      <c r="I83" s="43" t="inlineStr">
-        <is>
-          <t>Shodaqoh</t>
-        </is>
-      </c>
-      <c r="J83" s="44" t="n">
-        <v>50000</v>
-      </c>
+      <c r="A83" s="42" t="n"/>
+      <c r="B83" s="42" t="n"/>
+      <c r="C83" s="42" t="n"/>
+      <c r="D83" s="42" t="n"/>
+      <c r="E83" s="42" t="n"/>
+      <c r="F83" s="42" t="n"/>
+      <c r="G83" s="42" t="n"/>
+      <c r="H83" s="42" t="n"/>
+      <c r="I83" s="43" t="n"/>
+      <c r="J83" s="44" t="n"/>
       <c r="K83" s="10" t="n"/>
       <c r="L83" s="45" t="n"/>
     </row>
     <row r="84" ht="15" customHeight="1" s="16">
-      <c r="A84" s="42" t="n">
-        <v>79</v>
-      </c>
-      <c r="B84" s="42" t="inlineStr">
-        <is>
-          <t>2026-03-12</t>
-        </is>
-      </c>
-      <c r="C84" s="42" t="inlineStr">
-        <is>
-          <t>18:13</t>
-        </is>
-      </c>
-      <c r="D84" s="42" t="inlineStr">
-        <is>
-          <t>Lukman Hadi</t>
-        </is>
-      </c>
-      <c r="E84" s="42" t="inlineStr">
-        <is>
-          <t>Tipar Kidul</t>
-        </is>
-      </c>
-      <c r="F84" s="42" t="inlineStr">
-        <is>
-          <t>05</t>
-        </is>
-      </c>
-      <c r="G84" s="42" t="inlineStr">
-        <is>
-          <t>03</t>
-        </is>
-      </c>
-      <c r="H84" s="42" t="inlineStr">
-        <is>
-          <t>instansi</t>
-        </is>
-      </c>
-      <c r="I84" s="43" t="inlineStr">
-        <is>
-          <t>Infaq</t>
-        </is>
-      </c>
-      <c r="J84" s="44" t="n">
-        <v>20000</v>
-      </c>
+      <c r="A84" s="42" t="n"/>
+      <c r="B84" s="42" t="n"/>
+      <c r="C84" s="42" t="n"/>
+      <c r="D84" s="42" t="n"/>
+      <c r="E84" s="42" t="n"/>
+      <c r="F84" s="42" t="n"/>
+      <c r="G84" s="42" t="n"/>
+      <c r="H84" s="42" t="n"/>
+      <c r="I84" s="43" t="n"/>
+      <c r="J84" s="44" t="n"/>
       <c r="K84" s="10" t="n"/>
       <c r="L84" s="45" t="n"/>
     </row>
     <row r="85" ht="15" customHeight="1" s="16">
-      <c r="A85" s="42" t="n">
-        <v>80</v>
-      </c>
-      <c r="B85" s="42" t="inlineStr">
-        <is>
-          <t>2026-03-04</t>
-        </is>
-      </c>
-      <c r="C85" s="42" t="inlineStr">
-        <is>
-          <t>18:46</t>
-        </is>
-      </c>
-      <c r="D85" s="42" t="inlineStr">
-        <is>
-          <t>Maulana Eko</t>
-        </is>
-      </c>
-      <c r="E85" s="42" t="inlineStr">
-        <is>
-          <t>Tipar Kidul</t>
-        </is>
-      </c>
-      <c r="F85" s="42" t="inlineStr">
-        <is>
-          <t>05</t>
-        </is>
-      </c>
-      <c r="G85" s="42" t="inlineStr">
-        <is>
-          <t>03</t>
-        </is>
-      </c>
-      <c r="H85" s="42" t="inlineStr">
-        <is>
-          <t>instansi</t>
-        </is>
-      </c>
-      <c r="I85" s="43" t="inlineStr">
-        <is>
-          <t>Shodaqoh</t>
-        </is>
-      </c>
-      <c r="J85" s="44" t="n">
-        <v>50000</v>
-      </c>
+      <c r="A85" s="42" t="n"/>
+      <c r="B85" s="42" t="n"/>
+      <c r="C85" s="42" t="n"/>
+      <c r="D85" s="42" t="n"/>
+      <c r="E85" s="42" t="n"/>
+      <c r="F85" s="42" t="n"/>
+      <c r="G85" s="42" t="n"/>
+      <c r="H85" s="42" t="n"/>
+      <c r="I85" s="43" t="n"/>
+      <c r="J85" s="44" t="n"/>
       <c r="K85" s="10" t="n"/>
       <c r="L85" s="45" t="n"/>
     </row>
     <row r="86" ht="15" customHeight="1" s="16">
-      <c r="A86" s="42" t="n">
-        <v>81</v>
-      </c>
-      <c r="B86" s="42" t="inlineStr">
-        <is>
-          <t>2026-03-13</t>
-        </is>
-      </c>
-      <c r="C86" s="42" t="inlineStr">
-        <is>
-          <t>19:26</t>
-        </is>
-      </c>
-      <c r="D86" s="42" t="inlineStr">
-        <is>
-          <t>19:26</t>
-        </is>
-      </c>
-      <c r="E86" s="42" t="inlineStr">
-        <is>
-          <t>Ajibarang Wetan</t>
-        </is>
-      </c>
-      <c r="F86" s="42" t="inlineStr">
-        <is>
-          <t>09</t>
-        </is>
-      </c>
-      <c r="G86" s="42" t="inlineStr">
-        <is>
-          <t>01</t>
-        </is>
-      </c>
-      <c r="H86" s="42" t="inlineStr">
-        <is>
-          <t>perorangan</t>
-        </is>
-      </c>
-      <c r="I86" s="43" t="inlineStr">
-        <is>
-          <t>Infaq</t>
-        </is>
-      </c>
-      <c r="J86" s="44" t="n">
-        <v>100000</v>
-      </c>
+      <c r="A86" s="42" t="n"/>
+      <c r="B86" s="42" t="n"/>
+      <c r="C86" s="42" t="n"/>
+      <c r="D86" s="42" t="n"/>
+      <c r="E86" s="42" t="n"/>
+      <c r="F86" s="42" t="n"/>
+      <c r="G86" s="42" t="n"/>
+      <c r="H86" s="42" t="n"/>
+      <c r="I86" s="43" t="n"/>
+      <c r="J86" s="44" t="n"/>
       <c r="K86" s="10" t="n"/>
       <c r="L86" s="45" t="n"/>
     </row>

</xml_diff>